<commit_message>
086 Week 19/19 update
</commit_message>
<xml_diff>
--- a/data/WINTER_GOLF_2526.xlsx
+++ b/data/WINTER_GOLF_2526.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="105">
   <si>
     <t>WINTER GOLF 25/26 - THURSDAY SINGLES</t>
   </si>
@@ -63,6 +63,18 @@
   </si>
   <si>
     <t>22nd Jan 26</t>
+  </si>
+  <si>
+    <t>29th Jan 26</t>
+  </si>
+  <si>
+    <t>5th Feb 26</t>
+  </si>
+  <si>
+    <t>12th Feb 26</t>
+  </si>
+  <si>
+    <t>19th Feb 26</t>
   </si>
   <si>
     <t>NAME</t>
@@ -237,6 +249,18 @@
   </si>
   <si>
     <t>25th Jan 26</t>
+  </si>
+  <si>
+    <t>1st Feb 26</t>
+  </si>
+  <si>
+    <t>8th Feb 26</t>
+  </si>
+  <si>
+    <t>15th Feb 26</t>
+  </si>
+  <si>
+    <t>22nd Feb 26</t>
   </si>
   <si>
     <t>MICK SKINNER</t>
@@ -913,10 +937,18 @@
       <c r="Q3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="R3" s="4"/>
-      <c r="S3" s="3"/>
-      <c r="T3" s="4"/>
-      <c r="U3" s="3"/>
+      <c r="R3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="S3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="T3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="U3" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="V3" s="4"/>
       <c r="W3" s="3"/>
       <c r="X3" s="4"/>
@@ -926,87 +958,87 @@
     </row>
     <row r="4">
       <c r="B4" s="7" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="Q4" s="8" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R4" s="8" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="S4" s="8" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="T4" s="8" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="U4" s="8" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="V4" s="8" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="W4" s="8" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="X4" s="8" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="Y4" s="8" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="Z4" s="8" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="AA4" s="10" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="11" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="13">
@@ -1059,7 +1091,7 @@
     </row>
     <row r="6">
       <c r="B6" s="17" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C6" s="12">
         <v>28.0</v>
@@ -1094,7 +1126,9 @@
         <v>32.0</v>
       </c>
       <c r="Q6" s="12"/>
-      <c r="R6" s="13"/>
+      <c r="R6" s="13">
+        <v>29.0</v>
+      </c>
       <c r="S6" s="12"/>
       <c r="T6" s="13"/>
       <c r="U6" s="12"/>
@@ -1105,12 +1139,12 @@
       <c r="Z6" s="18"/>
       <c r="AA6" s="14">
         <f t="shared" si="1"/>
-        <v>258</v>
+        <v>287</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="17" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C7" s="12">
         <v>31.0</v>
@@ -1143,7 +1177,9 @@
       <c r="Q7" s="12">
         <v>34.0</v>
       </c>
-      <c r="R7" s="13"/>
+      <c r="R7" s="13">
+        <v>37.0</v>
+      </c>
       <c r="S7" s="12"/>
       <c r="T7" s="13"/>
       <c r="U7" s="12"/>
@@ -1154,12 +1190,12 @@
       <c r="Z7" s="18"/>
       <c r="AA7" s="14">
         <f t="shared" si="1"/>
-        <v>273</v>
+        <v>310</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="17" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C8" s="12">
         <v>31.0</v>
@@ -1206,7 +1242,7 @@
     </row>
     <row r="9">
       <c r="B9" s="17" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C9" s="12">
         <v>34.0</v>
@@ -1261,7 +1297,7 @@
     </row>
     <row r="10">
       <c r="B10" s="17" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C10" s="12">
         <v>21.0</v>
@@ -1286,7 +1322,9 @@
         <v>30.0</v>
       </c>
       <c r="Q10" s="12"/>
-      <c r="R10" s="14"/>
+      <c r="R10" s="13">
+        <v>36.0</v>
+      </c>
       <c r="S10" s="15"/>
       <c r="T10" s="13"/>
       <c r="U10" s="12"/>
@@ -1297,12 +1335,12 @@
       <c r="Z10" s="16"/>
       <c r="AA10" s="14">
         <f t="shared" si="1"/>
-        <v>119</v>
+        <v>155</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="17" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C11" s="12">
         <v>36.0</v>
@@ -1355,7 +1393,7 @@
     </row>
     <row r="12">
       <c r="B12" s="17" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C12" s="12">
         <v>35.0</v>
@@ -1406,7 +1444,7 @@
     </row>
     <row r="13">
       <c r="B13" s="17" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C13" s="12">
         <v>34.0</v>
@@ -1451,7 +1489,7 @@
     </row>
     <row r="14">
       <c r="B14" s="17" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C14" s="12">
         <v>33.0</v>
@@ -1492,7 +1530,9 @@
       <c r="Q14" s="12">
         <v>37.0</v>
       </c>
-      <c r="R14" s="13"/>
+      <c r="R14" s="13">
+        <v>38.0</v>
+      </c>
       <c r="S14" s="12"/>
       <c r="T14" s="14"/>
       <c r="U14" s="15"/>
@@ -1503,12 +1543,12 @@
       <c r="Z14" s="18"/>
       <c r="AA14" s="14">
         <f t="shared" si="1"/>
-        <v>379</v>
+        <v>417</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="17" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="13"/>
@@ -1547,7 +1587,9 @@
       <c r="Q15" s="12">
         <v>26.0</v>
       </c>
-      <c r="R15" s="14"/>
+      <c r="R15" s="13">
+        <v>33.0</v>
+      </c>
       <c r="S15" s="12"/>
       <c r="T15" s="13"/>
       <c r="U15" s="15"/>
@@ -1558,12 +1600,12 @@
       <c r="Z15" s="18"/>
       <c r="AA15" s="14">
         <f t="shared" si="1"/>
-        <v>328</v>
+        <v>361</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="19" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C16" s="18">
         <v>26.0</v>
@@ -1596,7 +1638,9 @@
       <c r="Q16" s="12">
         <v>32.0</v>
       </c>
-      <c r="R16" s="13"/>
+      <c r="R16" s="13">
+        <v>31.0</v>
+      </c>
       <c r="S16" s="15"/>
       <c r="T16" s="13"/>
       <c r="U16" s="12"/>
@@ -1607,12 +1651,12 @@
       <c r="Z16" s="16"/>
       <c r="AA16" s="14">
         <f t="shared" si="1"/>
-        <v>245</v>
+        <v>276</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="21" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C17" s="12">
         <v>31.0</v>
@@ -1645,7 +1689,9 @@
         <v>29.0</v>
       </c>
       <c r="Q17" s="12"/>
-      <c r="R17" s="15"/>
+      <c r="R17" s="12">
+        <v>32.0</v>
+      </c>
       <c r="S17" s="15"/>
       <c r="T17" s="12"/>
       <c r="U17" s="15"/>
@@ -1656,7 +1702,7 @@
       <c r="Z17" s="12"/>
       <c r="AA17" s="14">
         <f t="shared" si="1"/>
-        <v>257</v>
+        <v>289</v>
       </c>
     </row>
     <row r="18" ht="9.0" customHeight="1">
@@ -1687,57 +1733,65 @@
     </row>
     <row r="19" ht="72.0" customHeight="1">
       <c r="B19" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C19" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="D19" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="E19" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="F19" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="G19" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="H19" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="I19" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="J19" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="K19" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="C19" s="24" t="s">
-        <v>48</v>
-      </c>
-      <c r="D19" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="E19" s="24" t="s">
-        <v>45</v>
-      </c>
-      <c r="F19" s="24" t="s">
-        <v>46</v>
-      </c>
-      <c r="G19" s="24" t="s">
-        <v>52</v>
-      </c>
-      <c r="H19" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="I19" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="J19" s="24" t="s">
-        <v>49</v>
-      </c>
-      <c r="K19" s="24" t="s">
-        <v>51</v>
-      </c>
       <c r="L19" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="M19" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="N19" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="O19" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="M19" s="24" t="s">
-        <v>54</v>
-      </c>
-      <c r="N19" s="24" t="s">
-        <v>56</v>
-      </c>
-      <c r="O19" s="24" t="s">
-        <v>52</v>
-      </c>
       <c r="P19" s="24" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="Q19" s="24" t="s">
-        <v>51</v>
-      </c>
-      <c r="R19" s="24"/>
-      <c r="S19" s="24"/>
-      <c r="T19" s="24"/>
-      <c r="U19" s="24"/>
+        <v>55</v>
+      </c>
+      <c r="R19" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="S19" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="T19" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="U19" s="24" t="s">
+        <v>60</v>
+      </c>
       <c r="V19" s="24"/>
       <c r="W19" s="24"/>
       <c r="X19" s="24"/>
@@ -1747,7 +1801,7 @@
     </row>
     <row r="20">
       <c r="B20" s="26" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C20" s="27">
         <v>36.0</v>
@@ -1790,7 +1844,9 @@
       <c r="Q20" s="27">
         <v>37.0</v>
       </c>
-      <c r="R20" s="27"/>
+      <c r="R20" s="27">
+        <v>38.0</v>
+      </c>
       <c r="S20" s="27"/>
       <c r="T20" s="27"/>
       <c r="U20" s="27"/>
@@ -1820,61 +1876,69 @@
   <sheetData>
     <row r="2" ht="24.0" customHeight="1">
       <c r="B2" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="Z2" s="2"/>
       <c r="AA2" s="2"/>
     </row>
     <row r="3" ht="73.5" customHeight="1">
       <c r="C3" s="3" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="R3" s="4"/>
-      <c r="S3" s="3"/>
-      <c r="T3" s="4"/>
-      <c r="U3" s="3"/>
+        <v>77</v>
+      </c>
+      <c r="R3" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="S3" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T3" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="U3" s="3" t="s">
+        <v>81</v>
+      </c>
       <c r="V3" s="4"/>
       <c r="W3" s="3"/>
       <c r="X3" s="4"/>
@@ -1884,87 +1948,87 @@
     </row>
     <row r="4">
       <c r="B4" s="7" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="Q4" s="8" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R4" s="8" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="S4" s="8" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="T4" s="8" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="U4" s="8" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="V4" s="8" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="W4" s="8" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="X4" s="8" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="Y4" s="8" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="Z4" s="8" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="AA4" s="10" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="11" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="13"/>
@@ -2001,7 +2065,7 @@
     </row>
     <row r="6">
       <c r="B6" s="17" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="C6" s="12">
         <v>38.0</v>
@@ -2031,7 +2095,9 @@
       <c r="R6" s="13"/>
       <c r="S6" s="12"/>
       <c r="T6" s="13"/>
-      <c r="U6" s="12"/>
+      <c r="U6" s="12">
+        <v>33.0</v>
+      </c>
       <c r="V6" s="13"/>
       <c r="W6" s="12"/>
       <c r="X6" s="13"/>
@@ -2039,12 +2105,12 @@
       <c r="Z6" s="16"/>
       <c r="AA6" s="14">
         <f t="shared" si="1"/>
-        <v>188</v>
+        <v>221</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="17" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="13">
@@ -2081,10 +2147,14 @@
       <c r="Q7" s="12">
         <v>29.0</v>
       </c>
-      <c r="R7" s="13"/>
+      <c r="R7" s="13">
+        <v>28.0</v>
+      </c>
       <c r="S7" s="12"/>
       <c r="T7" s="13"/>
-      <c r="U7" s="15"/>
+      <c r="U7" s="12">
+        <v>32.0</v>
+      </c>
       <c r="V7" s="14"/>
       <c r="W7" s="15"/>
       <c r="X7" s="14"/>
@@ -2092,12 +2162,12 @@
       <c r="Z7" s="16"/>
       <c r="AA7" s="14">
         <f t="shared" si="1"/>
-        <v>285</v>
+        <v>345</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="17" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C8" s="12">
         <v>28.0</v>
@@ -2129,7 +2199,9 @@
       <c r="R8" s="13"/>
       <c r="S8" s="12"/>
       <c r="T8" s="14"/>
-      <c r="U8" s="12"/>
+      <c r="U8" s="12">
+        <v>34.0</v>
+      </c>
       <c r="V8" s="13"/>
       <c r="W8" s="12"/>
       <c r="X8" s="14"/>
@@ -2137,12 +2209,12 @@
       <c r="Z8" s="18"/>
       <c r="AA8" s="14">
         <f t="shared" si="1"/>
-        <v>181</v>
+        <v>215</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="17" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="13">
@@ -2172,7 +2244,9 @@
       <c r="R9" s="14"/>
       <c r="S9" s="15"/>
       <c r="T9" s="14"/>
-      <c r="U9" s="12"/>
+      <c r="U9" s="12">
+        <v>31.0</v>
+      </c>
       <c r="V9" s="13"/>
       <c r="W9" s="12"/>
       <c r="X9" s="13"/>
@@ -2180,12 +2254,12 @@
       <c r="Z9" s="16"/>
       <c r="AA9" s="14">
         <f t="shared" si="1"/>
-        <v>167</v>
+        <v>198</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="17" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C10" s="15"/>
       <c r="D10" s="13"/>
@@ -2230,7 +2304,7 @@
     </row>
     <row r="11">
       <c r="B11" s="17" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="C11" s="12">
         <v>33.0</v>
@@ -2257,7 +2331,9 @@
       <c r="Q11" s="12">
         <v>34.0</v>
       </c>
-      <c r="R11" s="14"/>
+      <c r="R11" s="13">
+        <v>35.0</v>
+      </c>
       <c r="S11" s="15"/>
       <c r="T11" s="14"/>
       <c r="U11" s="15"/>
@@ -2268,12 +2344,12 @@
       <c r="Z11" s="16"/>
       <c r="AA11" s="14">
         <f t="shared" si="1"/>
-        <v>175</v>
+        <v>210</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="17" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="13"/>
@@ -2301,7 +2377,9 @@
       <c r="R12" s="14"/>
       <c r="S12" s="12"/>
       <c r="T12" s="14"/>
-      <c r="U12" s="15"/>
+      <c r="U12" s="12">
+        <v>31.0</v>
+      </c>
       <c r="V12" s="14"/>
       <c r="W12" s="12"/>
       <c r="X12" s="13"/>
@@ -2309,12 +2387,12 @@
       <c r="Z12" s="18"/>
       <c r="AA12" s="14">
         <f t="shared" si="1"/>
-        <v>135</v>
+        <v>166</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="17" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="C13" s="12">
         <v>33.0</v>
@@ -2350,7 +2428,9 @@
       <c r="R13" s="14"/>
       <c r="S13" s="15"/>
       <c r="T13" s="13"/>
-      <c r="U13" s="12"/>
+      <c r="U13" s="12">
+        <v>36.0</v>
+      </c>
       <c r="V13" s="13"/>
       <c r="W13" s="12"/>
       <c r="X13" s="14"/>
@@ -2358,12 +2438,12 @@
       <c r="Z13" s="16"/>
       <c r="AA13" s="14">
         <f t="shared" si="1"/>
-        <v>235</v>
+        <v>271</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="17" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C14" s="12">
         <v>29.0</v>
@@ -2400,10 +2480,14 @@
       <c r="Q14" s="12">
         <v>26.0</v>
       </c>
-      <c r="R14" s="14"/>
+      <c r="R14" s="13">
+        <v>39.0</v>
+      </c>
       <c r="S14" s="15"/>
       <c r="T14" s="14"/>
-      <c r="U14" s="12"/>
+      <c r="U14" s="12">
+        <v>28.0</v>
+      </c>
       <c r="V14" s="13"/>
       <c r="W14" s="12"/>
       <c r="X14" s="13"/>
@@ -2411,12 +2495,12 @@
       <c r="Z14" s="16"/>
       <c r="AA14" s="14">
         <f t="shared" si="1"/>
-        <v>289</v>
+        <v>356</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="17" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C15" s="12">
         <v>28.0</v>
@@ -2451,10 +2535,14 @@
       <c r="Q15" s="12">
         <v>34.0</v>
       </c>
-      <c r="R15" s="14"/>
+      <c r="R15" s="13">
+        <v>22.0</v>
+      </c>
       <c r="S15" s="12"/>
       <c r="T15" s="14"/>
-      <c r="U15" s="15"/>
+      <c r="U15" s="12">
+        <v>31.0</v>
+      </c>
       <c r="V15" s="13"/>
       <c r="W15" s="12"/>
       <c r="X15" s="13"/>
@@ -2462,12 +2550,12 @@
       <c r="Z15" s="16"/>
       <c r="AA15" s="14">
         <f t="shared" si="1"/>
-        <v>267</v>
+        <v>320</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="17" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C16" s="12">
         <v>24.0</v>
@@ -2498,10 +2586,14 @@
       <c r="Q16" s="12">
         <v>32.0</v>
       </c>
-      <c r="R16" s="14"/>
+      <c r="R16" s="13">
+        <v>31.0</v>
+      </c>
       <c r="S16" s="12"/>
       <c r="T16" s="14"/>
-      <c r="U16" s="12"/>
+      <c r="U16" s="12">
+        <v>25.0</v>
+      </c>
       <c r="V16" s="13"/>
       <c r="W16" s="12"/>
       <c r="X16" s="13"/>
@@ -2509,12 +2601,12 @@
       <c r="Z16" s="16"/>
       <c r="AA16" s="14">
         <f t="shared" si="1"/>
-        <v>218</v>
+        <v>274</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="17" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="C17" s="12">
         <v>31.0</v>
@@ -2549,10 +2641,14 @@
       <c r="Q17" s="12">
         <v>31.0</v>
       </c>
-      <c r="R17" s="14"/>
+      <c r="R17" s="13">
+        <v>41.0</v>
+      </c>
       <c r="S17" s="12"/>
       <c r="T17" s="13"/>
-      <c r="U17" s="12"/>
+      <c r="U17" s="12">
+        <v>34.0</v>
+      </c>
       <c r="V17" s="13"/>
       <c r="W17" s="12"/>
       <c r="X17" s="13"/>
@@ -2560,12 +2656,12 @@
       <c r="Z17" s="16"/>
       <c r="AA17" s="14">
         <f t="shared" si="1"/>
-        <v>281</v>
+        <v>356</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="17" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="C18" s="12">
         <v>35.0</v>
@@ -2610,7 +2706,7 @@
     </row>
     <row r="19">
       <c r="B19" s="17" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="C19" s="12">
         <v>33.0</v>
@@ -2649,10 +2745,14 @@
       <c r="Q19" s="12">
         <v>28.0</v>
       </c>
-      <c r="R19" s="14"/>
+      <c r="R19" s="13">
+        <v>38.0</v>
+      </c>
       <c r="S19" s="12"/>
       <c r="T19" s="14"/>
-      <c r="U19" s="12"/>
+      <c r="U19" s="12">
+        <v>29.0</v>
+      </c>
       <c r="V19" s="13"/>
       <c r="W19" s="15"/>
       <c r="X19" s="13"/>
@@ -2660,12 +2760,12 @@
       <c r="Z19" s="16"/>
       <c r="AA19" s="14">
         <f t="shared" si="1"/>
-        <v>354</v>
+        <v>421</v>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="17" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="C20" s="12">
         <v>27.0</v>
@@ -2698,10 +2798,14 @@
       <c r="Q20" s="12">
         <v>31.0</v>
       </c>
-      <c r="R20" s="14"/>
+      <c r="R20" s="13">
+        <v>39.0</v>
+      </c>
       <c r="S20" s="12"/>
       <c r="T20" s="13"/>
-      <c r="U20" s="15"/>
+      <c r="U20" s="12">
+        <v>27.0</v>
+      </c>
       <c r="V20" s="13"/>
       <c r="W20" s="12"/>
       <c r="X20" s="14"/>
@@ -2709,12 +2813,12 @@
       <c r="Z20" s="18"/>
       <c r="AA20" s="14">
         <f t="shared" si="1"/>
-        <v>233</v>
+        <v>299</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="17" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="C21" s="12">
         <v>31.0</v>
@@ -2759,7 +2863,7 @@
     </row>
     <row r="22">
       <c r="B22" s="28" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C22" s="12"/>
       <c r="D22" s="13"/>
@@ -2789,7 +2893,9 @@
       <c r="R22" s="14"/>
       <c r="S22" s="15"/>
       <c r="T22" s="13"/>
-      <c r="U22" s="15"/>
+      <c r="U22" s="12">
+        <v>28.0</v>
+      </c>
       <c r="V22" s="13"/>
       <c r="W22" s="12"/>
       <c r="X22" s="13"/>
@@ -2797,7 +2903,7 @@
       <c r="Z22" s="18"/>
       <c r="AA22" s="14">
         <f t="shared" si="1"/>
-        <v>165</v>
+        <v>193</v>
       </c>
     </row>
     <row r="23" ht="9.0" customHeight="1">
@@ -2828,57 +2934,65 @@
     </row>
     <row r="24" ht="84.75" customHeight="1">
       <c r="B24" s="23" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C24" s="24" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="D24" s="24" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="E24" s="24" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F24" s="24" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G24" s="24" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="H24" s="24" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="I24" s="24" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="J24" s="24" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="K24" s="24" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="L24" s="24" t="s">
+        <v>94</v>
+      </c>
+      <c r="M24" s="24" t="s">
+        <v>82</v>
+      </c>
+      <c r="N24" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="O24" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="P24" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q24" s="24" t="s">
+        <v>94</v>
+      </c>
+      <c r="R24" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="S24" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="T24" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="U24" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="M24" s="24" t="s">
-        <v>74</v>
-      </c>
-      <c r="N24" s="24" t="s">
-        <v>56</v>
-      </c>
-      <c r="O24" s="24" t="s">
-        <v>56</v>
-      </c>
-      <c r="P24" s="24" t="s">
-        <v>56</v>
-      </c>
-      <c r="Q24" s="24" t="s">
-        <v>86</v>
-      </c>
-      <c r="R24" s="24"/>
-      <c r="S24" s="24"/>
-      <c r="T24" s="24"/>
-      <c r="U24" s="24"/>
       <c r="V24" s="24"/>
       <c r="W24" s="24"/>
       <c r="X24" s="24"/>
@@ -2888,7 +3002,7 @@
     </row>
     <row r="25">
       <c r="B25" s="26" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C25" s="27">
         <v>38.0</v>
@@ -2929,10 +3043,14 @@
       <c r="Q25" s="27">
         <v>36.0</v>
       </c>
-      <c r="R25" s="27"/>
+      <c r="R25" s="27">
+        <v>41.0</v>
+      </c>
       <c r="S25" s="27"/>
       <c r="T25" s="27"/>
-      <c r="U25" s="27"/>
+      <c r="U25" s="27">
+        <v>36.0</v>
+      </c>
       <c r="V25" s="27"/>
       <c r="W25" s="27"/>
       <c r="X25" s="27"/>
@@ -2959,18 +3077,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="30" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B1" s="31" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="C1" s="32" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="11" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="B2" s="33"/>
       <c r="C2" s="34">
@@ -2979,7 +3097,7 @@
     </row>
     <row r="3">
       <c r="A3" s="17" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B3" s="33"/>
       <c r="C3" s="34">
@@ -2988,7 +3106,7 @@
     </row>
     <row r="4">
       <c r="A4" s="17" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="B4" s="33"/>
       <c r="C4" s="34">
@@ -2997,7 +3115,7 @@
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="B5" s="33"/>
       <c r="C5" s="34">
@@ -3006,7 +3124,7 @@
     </row>
     <row r="6">
       <c r="A6" s="17" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="B6" s="33"/>
       <c r="C6" s="34">
@@ -3015,7 +3133,7 @@
     </row>
     <row r="7">
       <c r="A7" s="17" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="B7" s="33"/>
       <c r="C7" s="34">
@@ -3024,7 +3142,7 @@
     </row>
     <row r="8">
       <c r="A8" s="17" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B8" s="33"/>
       <c r="C8" s="34">
@@ -3033,25 +3151,25 @@
     </row>
     <row r="9">
       <c r="A9" s="17" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="B9" s="33"/>
       <c r="C9" s="34">
-        <v>11.0</v>
+        <v>10.0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="17" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="B10" s="33"/>
       <c r="C10" s="34">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="17" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B11" s="33"/>
       <c r="C11" s="34">
@@ -3060,7 +3178,7 @@
     </row>
     <row r="12">
       <c r="A12" s="17" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B12" s="33"/>
       <c r="C12" s="35">
@@ -3069,7 +3187,7 @@
     </row>
     <row r="13">
       <c r="A13" s="17" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B13" s="33"/>
       <c r="C13" s="34">
@@ -3078,7 +3196,7 @@
     </row>
     <row r="14">
       <c r="A14" s="17" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B14" s="33"/>
       <c r="C14" s="34">
@@ -3087,7 +3205,7 @@
     </row>
     <row r="15">
       <c r="A15" s="17" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B15" s="33"/>
       <c r="C15" s="34">
@@ -3096,16 +3214,16 @@
     </row>
     <row r="16">
       <c r="A16" s="17" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B16" s="33"/>
       <c r="C16" s="34">
-        <v>12.0</v>
+        <v>11.0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B17" s="33"/>
       <c r="C17" s="34">
@@ -3114,7 +3232,7 @@
     </row>
     <row r="18">
       <c r="A18" s="17" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="B18" s="33"/>
       <c r="C18" s="34">
@@ -3123,7 +3241,7 @@
     </row>
     <row r="19">
       <c r="A19" s="17" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="B19" s="33"/>
       <c r="C19" s="34">
@@ -3132,7 +3250,7 @@
     </row>
     <row r="20">
       <c r="A20" s="36" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B20" s="33"/>
       <c r="C20" s="34">
@@ -3141,7 +3259,7 @@
     </row>
     <row r="21">
       <c r="A21" s="17" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="B21" s="33"/>
       <c r="C21" s="34">
@@ -3150,7 +3268,7 @@
     </row>
     <row r="22">
       <c r="A22" s="17" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B22" s="33"/>
       <c r="C22" s="34">
@@ -3159,7 +3277,7 @@
     </row>
     <row r="23">
       <c r="A23" s="17" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B23" s="33"/>
       <c r="C23" s="34">
@@ -3168,7 +3286,7 @@
     </row>
     <row r="24">
       <c r="A24" s="28" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="B24" s="37"/>
       <c r="C24" s="38">
@@ -3177,7 +3295,7 @@
     </row>
     <row r="25">
       <c r="A25" s="36" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B25" s="14"/>
       <c r="C25" s="13">
@@ -7087,13 +7205,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="B1" s="39" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="C1" s="40" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2">
@@ -7101,10 +7219,10 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="42" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="C2" s="43" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3">
@@ -7112,10 +7230,10 @@
         <v>2.0</v>
       </c>
       <c r="B3" s="44" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C3" s="45" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4">
@@ -7123,10 +7241,10 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="44" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="C4" s="45" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5">
@@ -7134,10 +7252,10 @@
         <v>4.0</v>
       </c>
       <c r="B5" s="44" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C5" s="45" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6">
@@ -7145,10 +7263,10 @@
         <v>5.0</v>
       </c>
       <c r="B6" s="44" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C6" s="45" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7">
@@ -7156,10 +7274,10 @@
         <v>6.0</v>
       </c>
       <c r="B7" s="44" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C7" s="45" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8">
@@ -7167,10 +7285,10 @@
         <v>7.0</v>
       </c>
       <c r="B8" s="44" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C8" s="45" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9">
@@ -7178,10 +7296,10 @@
         <v>8.0</v>
       </c>
       <c r="B9" s="44" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C9" s="45" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10">
@@ -7189,10 +7307,10 @@
         <v>9.0</v>
       </c>
       <c r="B10" s="44" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" s="45" t="s">
         <v>56</v>
-      </c>
-      <c r="C10" s="45" t="s">
-        <v>52</v>
       </c>
       <c r="G10" s="14"/>
     </row>
@@ -7201,10 +7319,10 @@
         <v>10.0</v>
       </c>
       <c r="B11" s="44" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="C11" s="45" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12">
@@ -7212,10 +7330,10 @@
         <v>11.0</v>
       </c>
       <c r="B12" s="44" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C12" s="45" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13">
@@ -7223,10 +7341,10 @@
         <v>12.0</v>
       </c>
       <c r="B13" s="44" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C13" s="45" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14">
@@ -7234,10 +7352,10 @@
         <v>13.0</v>
       </c>
       <c r="B14" s="44" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C14" s="45" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15">
@@ -7245,10 +7363,10 @@
         <v>14.0</v>
       </c>
       <c r="B15" s="44" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C15" s="45" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16">
@@ -7256,39 +7374,55 @@
         <v>15.0</v>
       </c>
       <c r="B16" s="44" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C16" s="45" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="13">
         <v>16.0</v>
       </c>
-      <c r="B17" s="44"/>
-      <c r="C17" s="45"/>
+      <c r="B17" s="44" t="s">
+        <v>94</v>
+      </c>
+      <c r="C17" s="45" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="13">
         <v>17.0</v>
       </c>
-      <c r="B18" s="44"/>
-      <c r="C18" s="45"/>
+      <c r="B18" s="44" t="s">
+        <v>60</v>
+      </c>
+      <c r="C18" s="45" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="13">
         <v>18.0</v>
       </c>
-      <c r="B19" s="44"/>
-      <c r="C19" s="45"/>
+      <c r="B19" s="44" t="s">
+        <v>60</v>
+      </c>
+      <c r="C19" s="45" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="13">
         <v>19.0</v>
       </c>
-      <c r="B20" s="44"/>
-      <c r="C20" s="45"/>
+      <c r="B20" s="44" t="s">
+        <v>83</v>
+      </c>
+      <c r="C20" s="45" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="13">
@@ -12199,19 +12333,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="D1" s="46" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="E1" s="26" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2">
@@ -12535,19 +12669,19 @@
       </c>
       <c r="B17" s="47" t="str">
         <f>'SUNDAY SINGLES'!R24</f>
-        <v/>
-      </c>
-      <c r="C17" s="47" t="str">
+        <v>FRED HOLLINGWORTH</v>
+      </c>
+      <c r="C17" s="47">
         <f>'SUNDAY SINGLES'!R25</f>
-        <v/>
+        <v>41</v>
       </c>
       <c r="D17" s="48" t="str">
         <f>'THURSDAY SINGLES'!R19</f>
-        <v/>
-      </c>
-      <c r="E17" s="47" t="str">
+        <v>ALBIE GILLESPIE</v>
+      </c>
+      <c r="E17" s="47">
         <f>'THURSDAY SINGLES'!R20</f>
-        <v/>
+        <v>38</v>
       </c>
     </row>
     <row r="18">
@@ -12556,7 +12690,7 @@
       </c>
       <c r="B18" s="47" t="str">
         <f>'SUNDAY SINGLES'!S24</f>
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="C18" s="47" t="str">
         <f>'SUNDAY SINGLES'!S25</f>
@@ -12564,7 +12698,7 @@
       </c>
       <c r="D18" s="48" t="str">
         <f>'THURSDAY SINGLES'!S19</f>
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="E18" s="47" t="str">
         <f>'THURSDAY SINGLES'!S20</f>
@@ -12577,7 +12711,7 @@
       </c>
       <c r="B19" s="47" t="str">
         <f>'SUNDAY SINGLES'!T24</f>
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="C19" s="47" t="str">
         <f>'SUNDAY SINGLES'!T25</f>
@@ -12585,7 +12719,7 @@
       </c>
       <c r="D19" s="48" t="str">
         <f>'THURSDAY SINGLES'!T19</f>
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="E19" s="47" t="str">
         <f>'THURSDAY SINGLES'!T20</f>
@@ -12598,15 +12732,15 @@
       </c>
       <c r="B20" s="47" t="str">
         <f>'SUNDAY SINGLES'!U24</f>
-        <v/>
-      </c>
-      <c r="C20" s="47" t="str">
+        <v>STEVE FELLOWS</v>
+      </c>
+      <c r="C20" s="47">
         <f>'SUNDAY SINGLES'!U25</f>
-        <v/>
+        <v>36</v>
       </c>
       <c r="D20" s="48" t="str">
         <f>'THURSDAY SINGLES'!U19</f>
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="E20" s="47" t="str">
         <f>'THURSDAY SINGLES'!U20</f>

</xml_diff>

<commit_message>
087 Week 20/20 data update
</commit_message>
<xml_diff>
--- a/data/WINTER_GOLF_2526.xlsx
+++ b/data/WINTER_GOLF_2526.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="107">
   <si>
     <t>WINTER GOLF 25/26 - THURSDAY SINGLES</t>
   </si>
@@ -75,6 +75,9 @@
   </si>
   <si>
     <t>19th Feb 26</t>
+  </si>
+  <si>
+    <t>27th Feb 26</t>
   </si>
   <si>
     <t>NAME</t>
@@ -261,6 +264,9 @@
   </si>
   <si>
     <t>22nd Feb 26</t>
+  </si>
+  <si>
+    <t>1st March 26</t>
   </si>
   <si>
     <t>MICK SKINNER</t>
@@ -949,7 +955,9 @@
       <c r="U3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="V3" s="4"/>
+      <c r="V3" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="W3" s="3"/>
       <c r="X3" s="4"/>
       <c r="Y3" s="3"/>
@@ -958,87 +966,87 @@
     </row>
     <row r="4">
       <c r="B4" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q4" s="8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="R4" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S4" s="8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="T4" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="U4" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="V4" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="W4" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="X4" s="8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Y4" s="8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Z4" s="8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AA4" s="10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="11" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="13">
@@ -1079,19 +1087,21 @@
       <c r="S5" s="12"/>
       <c r="T5" s="13"/>
       <c r="U5" s="12"/>
-      <c r="V5" s="14"/>
+      <c r="V5" s="13">
+        <v>33.0</v>
+      </c>
       <c r="W5" s="15"/>
       <c r="X5" s="14"/>
       <c r="Y5" s="15"/>
       <c r="Z5" s="16"/>
       <c r="AA5" s="14">
         <f t="shared" ref="AA5:AA17" si="1">sum(C5:Z5)</f>
-        <v>299</v>
+        <v>332</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="17" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C6" s="12">
         <v>28.0</v>
@@ -1132,19 +1142,21 @@
       <c r="S6" s="12"/>
       <c r="T6" s="13"/>
       <c r="U6" s="12"/>
-      <c r="V6" s="13"/>
+      <c r="V6" s="13">
+        <v>31.0</v>
+      </c>
       <c r="W6" s="12"/>
       <c r="X6" s="13"/>
       <c r="Y6" s="12"/>
       <c r="Z6" s="18"/>
       <c r="AA6" s="14">
         <f t="shared" si="1"/>
-        <v>287</v>
+        <v>318</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C7" s="12">
         <v>31.0</v>
@@ -1183,19 +1195,21 @@
       <c r="S7" s="12"/>
       <c r="T7" s="13"/>
       <c r="U7" s="12"/>
-      <c r="V7" s="14"/>
+      <c r="V7" s="13">
+        <v>29.0</v>
+      </c>
       <c r="W7" s="12"/>
       <c r="X7" s="14"/>
       <c r="Y7" s="12"/>
       <c r="Z7" s="18"/>
       <c r="AA7" s="14">
         <f t="shared" si="1"/>
-        <v>310</v>
+        <v>339</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="17" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C8" s="12">
         <v>31.0</v>
@@ -1230,19 +1244,21 @@
       <c r="S8" s="12"/>
       <c r="T8" s="13"/>
       <c r="U8" s="12"/>
-      <c r="V8" s="14"/>
+      <c r="V8" s="13">
+        <v>29.0</v>
+      </c>
       <c r="W8" s="15"/>
       <c r="X8" s="13"/>
       <c r="Y8" s="12"/>
       <c r="Z8" s="16"/>
       <c r="AA8" s="14">
         <f t="shared" si="1"/>
-        <v>239</v>
+        <v>268</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="17" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C9" s="12">
         <v>34.0</v>
@@ -1297,7 +1313,7 @@
     </row>
     <row r="10">
       <c r="B10" s="17" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C10" s="12">
         <v>21.0</v>
@@ -1328,19 +1344,21 @@
       <c r="S10" s="15"/>
       <c r="T10" s="13"/>
       <c r="U10" s="12"/>
-      <c r="V10" s="13"/>
+      <c r="V10" s="13">
+        <v>41.0</v>
+      </c>
       <c r="W10" s="12"/>
       <c r="X10" s="13"/>
       <c r="Y10" s="12"/>
       <c r="Z10" s="16"/>
       <c r="AA10" s="14">
         <f t="shared" si="1"/>
-        <v>155</v>
+        <v>196</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="17" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C11" s="12">
         <v>36.0</v>
@@ -1381,19 +1399,21 @@
       <c r="S11" s="12"/>
       <c r="T11" s="13"/>
       <c r="U11" s="15"/>
-      <c r="V11" s="14"/>
+      <c r="V11" s="13">
+        <v>27.0</v>
+      </c>
       <c r="W11" s="15"/>
       <c r="X11" s="13"/>
       <c r="Y11" s="12"/>
       <c r="Z11" s="16"/>
       <c r="AA11" s="14">
         <f t="shared" si="1"/>
-        <v>277</v>
+        <v>304</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="17" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C12" s="12">
         <v>35.0</v>
@@ -1432,19 +1452,21 @@
       <c r="S12" s="12"/>
       <c r="T12" s="14"/>
       <c r="U12" s="15"/>
-      <c r="V12" s="13"/>
+      <c r="V12" s="13">
+        <v>29.0</v>
+      </c>
       <c r="W12" s="12"/>
       <c r="X12" s="13"/>
       <c r="Y12" s="12"/>
       <c r="Z12" s="18"/>
       <c r="AA12" s="14">
         <f t="shared" si="1"/>
-        <v>305</v>
+        <v>334</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="17" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C13" s="12">
         <v>34.0</v>
@@ -1477,19 +1499,21 @@
       <c r="S13" s="15"/>
       <c r="T13" s="13"/>
       <c r="U13" s="12"/>
-      <c r="V13" s="13"/>
+      <c r="V13" s="13">
+        <v>25.0</v>
+      </c>
       <c r="W13" s="12"/>
       <c r="X13" s="14"/>
       <c r="Y13" s="12"/>
       <c r="Z13" s="16"/>
       <c r="AA13" s="14">
         <f t="shared" si="1"/>
-        <v>168</v>
+        <v>193</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="17" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C14" s="12">
         <v>33.0</v>
@@ -1536,19 +1560,21 @@
       <c r="S14" s="12"/>
       <c r="T14" s="14"/>
       <c r="U14" s="15"/>
-      <c r="V14" s="13"/>
+      <c r="V14" s="13">
+        <v>36.0</v>
+      </c>
       <c r="W14" s="15"/>
       <c r="X14" s="13"/>
       <c r="Y14" s="12"/>
       <c r="Z14" s="18"/>
       <c r="AA14" s="14">
         <f t="shared" si="1"/>
-        <v>417</v>
+        <v>453</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="17" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="13"/>
@@ -1593,19 +1619,21 @@
       <c r="S15" s="12"/>
       <c r="T15" s="13"/>
       <c r="U15" s="15"/>
-      <c r="V15" s="14"/>
+      <c r="V15" s="13">
+        <v>37.0</v>
+      </c>
       <c r="W15" s="12"/>
       <c r="X15" s="13"/>
       <c r="Y15" s="12"/>
       <c r="Z15" s="18"/>
       <c r="AA15" s="14">
         <f t="shared" si="1"/>
-        <v>361</v>
+        <v>398</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="19" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C16" s="18">
         <v>26.0</v>
@@ -1656,7 +1684,7 @@
     </row>
     <row r="17">
       <c r="B17" s="21" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C17" s="12">
         <v>31.0</v>
@@ -1733,66 +1761,68 @@
     </row>
     <row r="19" ht="72.0" customHeight="1">
       <c r="B19" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="C19" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="D19" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="E19" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="F19" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="G19" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="H19" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="I19" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="J19" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="K19" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="L19" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="M19" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="C19" s="24" t="s">
+      <c r="N19" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="O19" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="P19" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q19" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="R19" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="S19" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="T19" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="U19" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="V19" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="D19" s="24" t="s">
-        <v>48</v>
-      </c>
-      <c r="E19" s="24" t="s">
-        <v>49</v>
-      </c>
-      <c r="F19" s="24" t="s">
-        <v>50</v>
-      </c>
-      <c r="G19" s="24" t="s">
-        <v>56</v>
-      </c>
-      <c r="H19" s="24" t="s">
-        <v>48</v>
-      </c>
-      <c r="I19" s="24" t="s">
-        <v>46</v>
-      </c>
-      <c r="J19" s="24" t="s">
-        <v>53</v>
-      </c>
-      <c r="K19" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="L19" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="M19" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="N19" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="O19" s="24" t="s">
-        <v>56</v>
-      </c>
-      <c r="P19" s="24" t="s">
-        <v>57</v>
-      </c>
-      <c r="Q19" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="R19" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="S19" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="T19" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="U19" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="V19" s="24"/>
       <c r="W19" s="24"/>
       <c r="X19" s="24"/>
       <c r="Y19" s="24"/>
@@ -1801,7 +1831,7 @@
     </row>
     <row r="20">
       <c r="B20" s="26" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C20" s="27">
         <v>36.0</v>
@@ -1850,7 +1880,9 @@
       <c r="S20" s="27"/>
       <c r="T20" s="27"/>
       <c r="U20" s="27"/>
-      <c r="V20" s="27"/>
+      <c r="V20" s="27">
+        <v>41.0</v>
+      </c>
       <c r="W20" s="27"/>
       <c r="X20" s="27"/>
       <c r="Y20" s="27"/>
@@ -1876,70 +1908,72 @@
   <sheetData>
     <row r="2" ht="24.0" customHeight="1">
       <c r="B2" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Z2" s="2"/>
       <c r="AA2" s="2"/>
     </row>
     <row r="3" ht="73.5" customHeight="1">
       <c r="C3" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="R3" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="S3" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="T3" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="U3" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="V3" s="4"/>
+        <v>82</v>
+      </c>
+      <c r="V3" s="4" t="s">
+        <v>83</v>
+      </c>
       <c r="W3" s="3"/>
       <c r="X3" s="4"/>
       <c r="Y3" s="3"/>
@@ -1948,87 +1982,87 @@
     </row>
     <row r="4">
       <c r="B4" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q4" s="8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="R4" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S4" s="8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="T4" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="U4" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="V4" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="W4" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="X4" s="8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Y4" s="8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Z4" s="8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AA4" s="10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="13"/>
@@ -2065,7 +2099,7 @@
     </row>
     <row r="6">
       <c r="B6" s="17" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C6" s="12">
         <v>38.0</v>
@@ -2110,7 +2144,7 @@
     </row>
     <row r="7">
       <c r="B7" s="17" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="13">
@@ -2167,7 +2201,7 @@
     </row>
     <row r="8">
       <c r="B8" s="17" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C8" s="12">
         <v>28.0</v>
@@ -2214,7 +2248,7 @@
     </row>
     <row r="9">
       <c r="B9" s="17" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="13">
@@ -2259,7 +2293,7 @@
     </row>
     <row r="10">
       <c r="B10" s="17" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C10" s="15"/>
       <c r="D10" s="13"/>
@@ -2304,7 +2338,7 @@
     </row>
     <row r="11">
       <c r="B11" s="17" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C11" s="12">
         <v>33.0</v>
@@ -2349,7 +2383,7 @@
     </row>
     <row r="12">
       <c r="B12" s="17" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="13"/>
@@ -2392,7 +2426,7 @@
     </row>
     <row r="13">
       <c r="B13" s="17" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C13" s="12">
         <v>33.0</v>
@@ -2443,7 +2477,7 @@
     </row>
     <row r="14">
       <c r="B14" s="17" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C14" s="12">
         <v>29.0</v>
@@ -2500,7 +2534,7 @@
     </row>
     <row r="15">
       <c r="B15" s="17" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C15" s="12">
         <v>28.0</v>
@@ -2555,7 +2589,7 @@
     </row>
     <row r="16">
       <c r="B16" s="17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C16" s="12">
         <v>24.0</v>
@@ -2606,7 +2640,7 @@
     </row>
     <row r="17">
       <c r="B17" s="17" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C17" s="12">
         <v>31.0</v>
@@ -2661,7 +2695,7 @@
     </row>
     <row r="18">
       <c r="B18" s="17" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C18" s="12">
         <v>35.0</v>
@@ -2706,7 +2740,7 @@
     </row>
     <row r="19">
       <c r="B19" s="17" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C19" s="12">
         <v>33.0</v>
@@ -2765,7 +2799,7 @@
     </row>
     <row r="20">
       <c r="B20" s="17" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C20" s="12">
         <v>27.0</v>
@@ -2818,7 +2852,7 @@
     </row>
     <row r="21">
       <c r="B21" s="17" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C21" s="12">
         <v>31.0</v>
@@ -2863,7 +2897,7 @@
     </row>
     <row r="22">
       <c r="B22" s="28" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C22" s="12"/>
       <c r="D22" s="13"/>
@@ -2934,66 +2968,68 @@
     </row>
     <row r="24" ht="84.75" customHeight="1">
       <c r="B24" s="23" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C24" s="24" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D24" s="24" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E24" s="24" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F24" s="24" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G24" s="24" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H24" s="24" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="I24" s="24" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J24" s="24" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="K24" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="L24" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="M24" s="24" t="s">
+        <v>84</v>
+      </c>
+      <c r="N24" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="O24" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="P24" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q24" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="R24" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="L24" s="24" t="s">
-        <v>94</v>
-      </c>
-      <c r="M24" s="24" t="s">
-        <v>82</v>
-      </c>
-      <c r="N24" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="O24" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="P24" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q24" s="24" t="s">
-        <v>94</v>
-      </c>
-      <c r="R24" s="24" t="s">
-        <v>87</v>
-      </c>
       <c r="S24" s="24" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="T24" s="24" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="U24" s="24" t="s">
-        <v>86</v>
-      </c>
-      <c r="V24" s="24"/>
+        <v>88</v>
+      </c>
+      <c r="V24" s="24" t="s">
+        <v>61</v>
+      </c>
       <c r="W24" s="24"/>
       <c r="X24" s="24"/>
       <c r="Y24" s="24"/>
@@ -3002,7 +3038,7 @@
     </row>
     <row r="25">
       <c r="B25" s="26" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C25" s="27">
         <v>38.0</v>
@@ -3077,18 +3113,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="30" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B1" s="31" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C1" s="32" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="11" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B2" s="33"/>
       <c r="C2" s="34">
@@ -3097,7 +3133,7 @@
     </row>
     <row r="3">
       <c r="A3" s="17" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B3" s="33"/>
       <c r="C3" s="34">
@@ -3106,7 +3142,7 @@
     </row>
     <row r="4">
       <c r="A4" s="17" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B4" s="33"/>
       <c r="C4" s="34">
@@ -3115,7 +3151,7 @@
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B5" s="33"/>
       <c r="C5" s="34">
@@ -3124,7 +3160,7 @@
     </row>
     <row r="6">
       <c r="A6" s="17" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B6" s="33"/>
       <c r="C6" s="34">
@@ -3133,16 +3169,16 @@
     </row>
     <row r="7">
       <c r="A7" s="17" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B7" s="33"/>
       <c r="C7" s="34">
-        <v>11.0</v>
+        <v>10.0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="17" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B8" s="33"/>
       <c r="C8" s="34">
@@ -3151,7 +3187,7 @@
     </row>
     <row r="9">
       <c r="A9" s="17" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B9" s="33"/>
       <c r="C9" s="34">
@@ -3160,7 +3196,7 @@
     </row>
     <row r="10">
       <c r="A10" s="17" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B10" s="33"/>
       <c r="C10" s="34">
@@ -3169,7 +3205,7 @@
     </row>
     <row r="11">
       <c r="A11" s="17" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B11" s="33"/>
       <c r="C11" s="34">
@@ -3178,7 +3214,7 @@
     </row>
     <row r="12">
       <c r="A12" s="17" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B12" s="33"/>
       <c r="C12" s="35">
@@ -3187,16 +3223,16 @@
     </row>
     <row r="13">
       <c r="A13" s="17" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B13" s="33"/>
       <c r="C13" s="34">
-        <v>28.0</v>
+        <v>25.0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="17" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B14" s="33"/>
       <c r="C14" s="34">
@@ -3205,7 +3241,7 @@
     </row>
     <row r="15">
       <c r="A15" s="17" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B15" s="33"/>
       <c r="C15" s="34">
@@ -3214,7 +3250,7 @@
     </row>
     <row r="16">
       <c r="A16" s="17" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B16" s="33"/>
       <c r="C16" s="34">
@@ -3223,16 +3259,16 @@
     </row>
     <row r="17">
       <c r="A17" s="17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B17" s="33"/>
       <c r="C17" s="34">
-        <v>9.0</v>
+        <v>10.0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="17" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B18" s="33"/>
       <c r="C18" s="34">
@@ -3241,7 +3277,7 @@
     </row>
     <row r="19">
       <c r="A19" s="17" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B19" s="33"/>
       <c r="C19" s="34">
@@ -3250,7 +3286,7 @@
     </row>
     <row r="20">
       <c r="A20" s="36" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B20" s="33"/>
       <c r="C20" s="34">
@@ -3259,7 +3295,7 @@
     </row>
     <row r="21">
       <c r="A21" s="17" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B21" s="33"/>
       <c r="C21" s="34">
@@ -3268,7 +3304,7 @@
     </row>
     <row r="22">
       <c r="A22" s="17" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B22" s="33"/>
       <c r="C22" s="34">
@@ -3277,7 +3313,7 @@
     </row>
     <row r="23">
       <c r="A23" s="17" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B23" s="33"/>
       <c r="C23" s="34">
@@ -3286,7 +3322,7 @@
     </row>
     <row r="24">
       <c r="A24" s="28" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B24" s="37"/>
       <c r="C24" s="38">
@@ -3295,7 +3331,7 @@
     </row>
     <row r="25">
       <c r="A25" s="36" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B25" s="14"/>
       <c r="C25" s="13">
@@ -7205,13 +7241,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B1" s="39" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C1" s="40" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2">
@@ -7219,10 +7255,10 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="42" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C2" s="43" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3">
@@ -7230,10 +7266,10 @@
         <v>2.0</v>
       </c>
       <c r="B3" s="44" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C3" s="45" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4">
@@ -7241,10 +7277,10 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="44" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C4" s="45" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
@@ -7252,10 +7288,10 @@
         <v>4.0</v>
       </c>
       <c r="B5" s="44" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C5" s="45" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6">
@@ -7263,10 +7299,10 @@
         <v>5.0</v>
       </c>
       <c r="B6" s="44" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C6" s="45" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7">
@@ -7274,10 +7310,10 @@
         <v>6.0</v>
       </c>
       <c r="B7" s="44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C7" s="45" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8">
@@ -7285,10 +7321,10 @@
         <v>7.0</v>
       </c>
       <c r="B8" s="44" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C8" s="45" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9">
@@ -7296,10 +7332,10 @@
         <v>8.0</v>
       </c>
       <c r="B9" s="44" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C9" s="45" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10">
@@ -7307,10 +7343,10 @@
         <v>9.0</v>
       </c>
       <c r="B10" s="44" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C10" s="45" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G10" s="14"/>
     </row>
@@ -7319,10 +7355,10 @@
         <v>10.0</v>
       </c>
       <c r="B11" s="44" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C11" s="45" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12">
@@ -7330,10 +7366,10 @@
         <v>11.0</v>
       </c>
       <c r="B12" s="44" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C12" s="45" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13">
@@ -7341,10 +7377,10 @@
         <v>12.0</v>
       </c>
       <c r="B13" s="44" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C13" s="45" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14">
@@ -7352,10 +7388,10 @@
         <v>13.0</v>
       </c>
       <c r="B14" s="44" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C14" s="45" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15">
@@ -7363,10 +7399,10 @@
         <v>14.0</v>
       </c>
       <c r="B15" s="44" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C15" s="45" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="16">
@@ -7374,10 +7410,10 @@
         <v>15.0</v>
       </c>
       <c r="B16" s="44" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C16" s="45" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="17">
@@ -7385,10 +7421,10 @@
         <v>16.0</v>
       </c>
       <c r="B17" s="44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C17" s="45" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="18">
@@ -7396,10 +7432,10 @@
         <v>17.0</v>
       </c>
       <c r="B18" s="44" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C18" s="45" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="19">
@@ -7407,10 +7443,10 @@
         <v>18.0</v>
       </c>
       <c r="B19" s="44" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C19" s="45" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20">
@@ -7418,18 +7454,22 @@
         <v>19.0</v>
       </c>
       <c r="B20" s="44" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C20" s="45" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="13">
         <v>20.0</v>
       </c>
-      <c r="B21" s="44"/>
-      <c r="C21" s="45"/>
+      <c r="B21" s="44" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" s="45" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="13">
@@ -12333,19 +12373,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D1" s="46" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E1" s="26" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2">
@@ -12753,7 +12793,7 @@
       </c>
       <c r="B21" s="47" t="str">
         <f>'SUNDAY SINGLES'!V24</f>
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="C21" s="47" t="str">
         <f>'SUNDAY SINGLES'!V25</f>
@@ -12761,11 +12801,11 @@
       </c>
       <c r="D21" s="48" t="str">
         <f>'THURSDAY SINGLES'!V19</f>
-        <v/>
-      </c>
-      <c r="E21" s="47" t="str">
+        <v>JOHN KING</v>
+      </c>
+      <c r="E21" s="47">
         <f>'THURSDAY SINGLES'!V20</f>
-        <v/>
+        <v>41</v>
       </c>
     </row>
     <row r="22">

</xml_diff>

<commit_message>
088 Week 21/21 data update
</commit_message>
<xml_diff>
--- a/data/WINTER_GOLF_2526.xlsx
+++ b/data/WINTER_GOLF_2526.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="109">
   <si>
     <t>WINTER GOLF 25/26 - THURSDAY SINGLES</t>
   </si>
@@ -78,6 +78,9 @@
   </si>
   <si>
     <t>27th Feb 26</t>
+  </si>
+  <si>
+    <t>5th March 26</t>
   </si>
   <si>
     <t>NAME</t>
@@ -267,6 +270,9 @@
   </si>
   <si>
     <t>1st March 26</t>
+  </si>
+  <si>
+    <t>8th March 26</t>
   </si>
   <si>
     <t>MICK SKINNER</t>
@@ -958,7 +964,9 @@
       <c r="V3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="W3" s="3"/>
+      <c r="W3" s="3" t="s">
+        <v>21</v>
+      </c>
       <c r="X3" s="4"/>
       <c r="Y3" s="3"/>
       <c r="Z3" s="5"/>
@@ -966,87 +974,87 @@
     </row>
     <row r="4">
       <c r="B4" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q4" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R4" s="8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="S4" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="T4" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="U4" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="V4" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="W4" s="8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="X4" s="8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Y4" s="8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Z4" s="8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AA4" s="10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="11" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="13">
@@ -1090,18 +1098,20 @@
       <c r="V5" s="13">
         <v>33.0</v>
       </c>
-      <c r="W5" s="15"/>
+      <c r="W5" s="12">
+        <v>39.0</v>
+      </c>
       <c r="X5" s="14"/>
       <c r="Y5" s="15"/>
       <c r="Z5" s="16"/>
       <c r="AA5" s="14">
         <f t="shared" ref="AA5:AA17" si="1">sum(C5:Z5)</f>
-        <v>332</v>
+        <v>371</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C6" s="12">
         <v>28.0</v>
@@ -1145,18 +1155,20 @@
       <c r="V6" s="13">
         <v>31.0</v>
       </c>
-      <c r="W6" s="12"/>
+      <c r="W6" s="12">
+        <v>35.0</v>
+      </c>
       <c r="X6" s="13"/>
       <c r="Y6" s="12"/>
       <c r="Z6" s="18"/>
       <c r="AA6" s="14">
         <f t="shared" si="1"/>
-        <v>318</v>
+        <v>353</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="17" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C7" s="12">
         <v>31.0</v>
@@ -1198,18 +1210,20 @@
       <c r="V7" s="13">
         <v>29.0</v>
       </c>
-      <c r="W7" s="12"/>
+      <c r="W7" s="12">
+        <v>36.0</v>
+      </c>
       <c r="X7" s="14"/>
       <c r="Y7" s="12"/>
       <c r="Z7" s="18"/>
       <c r="AA7" s="14">
         <f t="shared" si="1"/>
-        <v>339</v>
+        <v>375</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="17" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C8" s="12">
         <v>31.0</v>
@@ -1247,18 +1261,20 @@
       <c r="V8" s="13">
         <v>29.0</v>
       </c>
-      <c r="W8" s="15"/>
+      <c r="W8" s="12">
+        <v>32.0</v>
+      </c>
       <c r="X8" s="13"/>
       <c r="Y8" s="12"/>
       <c r="Z8" s="16"/>
       <c r="AA8" s="14">
         <f t="shared" si="1"/>
-        <v>268</v>
+        <v>300</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="17" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C9" s="12">
         <v>34.0</v>
@@ -1302,18 +1318,20 @@
       <c r="T9" s="13"/>
       <c r="U9" s="12"/>
       <c r="V9" s="14"/>
-      <c r="W9" s="15"/>
+      <c r="W9" s="12">
+        <v>28.0</v>
+      </c>
       <c r="X9" s="14"/>
       <c r="Y9" s="15"/>
       <c r="Z9" s="16"/>
       <c r="AA9" s="14">
         <f t="shared" si="1"/>
-        <v>332</v>
+        <v>360</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="17" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C10" s="12">
         <v>21.0</v>
@@ -1358,7 +1376,7 @@
     </row>
     <row r="11">
       <c r="B11" s="17" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C11" s="12">
         <v>36.0</v>
@@ -1402,18 +1420,20 @@
       <c r="V11" s="13">
         <v>27.0</v>
       </c>
-      <c r="W11" s="15"/>
+      <c r="W11" s="12">
+        <v>30.0</v>
+      </c>
       <c r="X11" s="13"/>
       <c r="Y11" s="12"/>
       <c r="Z11" s="16"/>
       <c r="AA11" s="14">
         <f t="shared" si="1"/>
-        <v>304</v>
+        <v>334</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="17" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C12" s="12">
         <v>35.0</v>
@@ -1466,7 +1486,7 @@
     </row>
     <row r="13">
       <c r="B13" s="17" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C13" s="12">
         <v>34.0</v>
@@ -1513,7 +1533,7 @@
     </row>
     <row r="14">
       <c r="B14" s="17" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C14" s="12">
         <v>33.0</v>
@@ -1563,18 +1583,20 @@
       <c r="V14" s="13">
         <v>36.0</v>
       </c>
-      <c r="W14" s="15"/>
+      <c r="W14" s="12">
+        <v>41.0</v>
+      </c>
       <c r="X14" s="13"/>
       <c r="Y14" s="12"/>
       <c r="Z14" s="18"/>
       <c r="AA14" s="14">
         <f t="shared" si="1"/>
-        <v>453</v>
+        <v>494</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="17" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="13"/>
@@ -1622,18 +1644,20 @@
       <c r="V15" s="13">
         <v>37.0</v>
       </c>
-      <c r="W15" s="12"/>
+      <c r="W15" s="12">
+        <v>30.0</v>
+      </c>
       <c r="X15" s="13"/>
       <c r="Y15" s="12"/>
       <c r="Z15" s="18"/>
       <c r="AA15" s="14">
         <f t="shared" si="1"/>
-        <v>398</v>
+        <v>428</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="19" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C16" s="18">
         <v>26.0</v>
@@ -1684,7 +1708,7 @@
     </row>
     <row r="17">
       <c r="B17" s="21" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C17" s="12">
         <v>31.0</v>
@@ -1724,13 +1748,15 @@
       <c r="T17" s="12"/>
       <c r="U17" s="15"/>
       <c r="V17" s="15"/>
-      <c r="W17" s="12"/>
+      <c r="W17" s="12">
+        <v>39.0</v>
+      </c>
       <c r="X17" s="12"/>
       <c r="Y17" s="12"/>
       <c r="Z17" s="12"/>
       <c r="AA17" s="14">
         <f t="shared" si="1"/>
-        <v>289</v>
+        <v>328</v>
       </c>
     </row>
     <row r="18" ht="9.0" customHeight="1">
@@ -1761,69 +1787,71 @@
     </row>
     <row r="19" ht="72.0" customHeight="1">
       <c r="B19" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="C19" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="E19" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="F19" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="G19" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="H19" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="I19" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="J19" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="K19" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="L19" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="M19" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="C19" s="24" t="s">
+      <c r="N19" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="O19" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="P19" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q19" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="R19" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="S19" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="T19" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="U19" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="V19" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="D19" s="24" t="s">
-        <v>49</v>
-      </c>
-      <c r="E19" s="24" t="s">
-        <v>50</v>
-      </c>
-      <c r="F19" s="24" t="s">
-        <v>51</v>
-      </c>
-      <c r="G19" s="24" t="s">
+      <c r="W19" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="H19" s="24" t="s">
-        <v>49</v>
-      </c>
-      <c r="I19" s="24" t="s">
-        <v>47</v>
-      </c>
-      <c r="J19" s="24" t="s">
-        <v>54</v>
-      </c>
-      <c r="K19" s="24" t="s">
-        <v>56</v>
-      </c>
-      <c r="L19" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="M19" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="N19" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="O19" s="24" t="s">
-        <v>57</v>
-      </c>
-      <c r="P19" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q19" s="24" t="s">
-        <v>56</v>
-      </c>
-      <c r="R19" s="24" t="s">
-        <v>56</v>
-      </c>
-      <c r="S19" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="T19" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="U19" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="V19" s="24" t="s">
-        <v>52</v>
-      </c>
-      <c r="W19" s="24"/>
       <c r="X19" s="24"/>
       <c r="Y19" s="24"/>
       <c r="Z19" s="24"/>
@@ -1831,7 +1859,7 @@
     </row>
     <row r="20">
       <c r="B20" s="26" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C20" s="27">
         <v>36.0</v>
@@ -1883,7 +1911,9 @@
       <c r="V20" s="27">
         <v>41.0</v>
       </c>
-      <c r="W20" s="27"/>
+      <c r="W20" s="27">
+        <v>41.0</v>
+      </c>
       <c r="X20" s="27"/>
       <c r="Y20" s="27"/>
       <c r="Z20" s="27"/>
@@ -1908,73 +1938,75 @@
   <sheetData>
     <row r="2" ht="24.0" customHeight="1">
       <c r="B2" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Z2" s="2"/>
       <c r="AA2" s="2"/>
     </row>
     <row r="3" ht="73.5" customHeight="1">
       <c r="C3" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="R3" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="S3" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="T3" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="U3" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="V3" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="W3" s="3"/>
+        <v>84</v>
+      </c>
+      <c r="W3" s="3" t="s">
+        <v>85</v>
+      </c>
       <c r="X3" s="4"/>
       <c r="Y3" s="3"/>
       <c r="Z3" s="5"/>
@@ -1982,87 +2014,87 @@
     </row>
     <row r="4">
       <c r="B4" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q4" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R4" s="8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="S4" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="T4" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="U4" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="V4" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="W4" s="8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="X4" s="8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Y4" s="8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Z4" s="8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AA4" s="10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="13"/>
@@ -2099,7 +2131,7 @@
     </row>
     <row r="6">
       <c r="B6" s="17" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C6" s="12">
         <v>38.0</v>
@@ -2133,18 +2165,20 @@
         <v>33.0</v>
       </c>
       <c r="V6" s="13"/>
-      <c r="W6" s="12"/>
+      <c r="W6" s="12">
+        <v>38.0</v>
+      </c>
       <c r="X6" s="13"/>
       <c r="Y6" s="12"/>
       <c r="Z6" s="16"/>
       <c r="AA6" s="14">
         <f t="shared" si="1"/>
-        <v>221</v>
+        <v>259</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="17" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="13">
@@ -2190,18 +2224,20 @@
         <v>32.0</v>
       </c>
       <c r="V7" s="14"/>
-      <c r="W7" s="15"/>
+      <c r="W7" s="12">
+        <v>34.0</v>
+      </c>
       <c r="X7" s="14"/>
       <c r="Y7" s="15"/>
       <c r="Z7" s="16"/>
       <c r="AA7" s="14">
         <f t="shared" si="1"/>
-        <v>345</v>
+        <v>379</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="17" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C8" s="12">
         <v>28.0</v>
@@ -2237,18 +2273,20 @@
         <v>34.0</v>
       </c>
       <c r="V8" s="13"/>
-      <c r="W8" s="12"/>
+      <c r="W8" s="12">
+        <v>36.0</v>
+      </c>
       <c r="X8" s="14"/>
       <c r="Y8" s="12"/>
       <c r="Z8" s="18"/>
       <c r="AA8" s="14">
         <f t="shared" si="1"/>
-        <v>215</v>
+        <v>251</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="17" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="13">
@@ -2282,18 +2320,20 @@
         <v>31.0</v>
       </c>
       <c r="V9" s="13"/>
-      <c r="W9" s="12"/>
+      <c r="W9" s="12">
+        <v>34.0</v>
+      </c>
       <c r="X9" s="13"/>
       <c r="Y9" s="15"/>
       <c r="Z9" s="16"/>
       <c r="AA9" s="14">
         <f t="shared" si="1"/>
-        <v>198</v>
+        <v>232</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="17" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C10" s="15"/>
       <c r="D10" s="13"/>
@@ -2327,18 +2367,20 @@
       <c r="T10" s="13"/>
       <c r="U10" s="12"/>
       <c r="V10" s="13"/>
-      <c r="W10" s="12"/>
+      <c r="W10" s="12">
+        <v>37.0</v>
+      </c>
       <c r="X10" s="13"/>
       <c r="Y10" s="15"/>
       <c r="Z10" s="16"/>
       <c r="AA10" s="14">
         <f t="shared" si="1"/>
-        <v>194</v>
+        <v>231</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="17" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C11" s="12">
         <v>33.0</v>
@@ -2383,7 +2425,7 @@
     </row>
     <row r="12">
       <c r="B12" s="17" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="13"/>
@@ -2426,7 +2468,7 @@
     </row>
     <row r="13">
       <c r="B13" s="17" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C13" s="12">
         <v>33.0</v>
@@ -2466,18 +2508,20 @@
         <v>36.0</v>
       </c>
       <c r="V13" s="13"/>
-      <c r="W13" s="12"/>
+      <c r="W13" s="12">
+        <v>28.0</v>
+      </c>
       <c r="X13" s="14"/>
       <c r="Y13" s="12"/>
       <c r="Z13" s="16"/>
       <c r="AA13" s="14">
         <f t="shared" si="1"/>
-        <v>271</v>
+        <v>299</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C14" s="12">
         <v>29.0</v>
@@ -2534,7 +2578,7 @@
     </row>
     <row r="15">
       <c r="B15" s="17" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C15" s="12">
         <v>28.0</v>
@@ -2589,7 +2633,7 @@
     </row>
     <row r="16">
       <c r="B16" s="17" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C16" s="12">
         <v>24.0</v>
@@ -2629,18 +2673,20 @@
         <v>25.0</v>
       </c>
       <c r="V16" s="13"/>
-      <c r="W16" s="12"/>
+      <c r="W16" s="12">
+        <v>27.0</v>
+      </c>
       <c r="X16" s="13"/>
       <c r="Y16" s="12"/>
       <c r="Z16" s="16"/>
       <c r="AA16" s="14">
         <f t="shared" si="1"/>
-        <v>274</v>
+        <v>301</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="17" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C17" s="12">
         <v>31.0</v>
@@ -2684,18 +2730,20 @@
         <v>34.0</v>
       </c>
       <c r="V17" s="13"/>
-      <c r="W17" s="12"/>
+      <c r="W17" s="12">
+        <v>36.0</v>
+      </c>
       <c r="X17" s="13"/>
       <c r="Y17" s="12"/>
       <c r="Z17" s="16"/>
       <c r="AA17" s="14">
         <f t="shared" si="1"/>
-        <v>356</v>
+        <v>392</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="17" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C18" s="12">
         <v>35.0</v>
@@ -2729,18 +2777,20 @@
       <c r="T18" s="13"/>
       <c r="U18" s="12"/>
       <c r="V18" s="13"/>
-      <c r="W18" s="12"/>
+      <c r="W18" s="12">
+        <v>37.0</v>
+      </c>
       <c r="X18" s="13"/>
       <c r="Y18" s="12"/>
       <c r="Z18" s="18"/>
       <c r="AA18" s="14">
         <f t="shared" si="1"/>
-        <v>196</v>
+        <v>233</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="17" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C19" s="12">
         <v>33.0</v>
@@ -2788,18 +2838,20 @@
         <v>29.0</v>
       </c>
       <c r="V19" s="13"/>
-      <c r="W19" s="15"/>
+      <c r="W19" s="12">
+        <v>32.0</v>
+      </c>
       <c r="X19" s="13"/>
       <c r="Y19" s="12"/>
       <c r="Z19" s="16"/>
       <c r="AA19" s="14">
         <f t="shared" si="1"/>
-        <v>421</v>
+        <v>453</v>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="17" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C20" s="12">
         <v>27.0</v>
@@ -2841,18 +2893,20 @@
         <v>27.0</v>
       </c>
       <c r="V20" s="13"/>
-      <c r="W20" s="12"/>
+      <c r="W20" s="12">
+        <v>30.0</v>
+      </c>
       <c r="X20" s="14"/>
       <c r="Y20" s="12"/>
       <c r="Z20" s="18"/>
       <c r="AA20" s="14">
         <f t="shared" si="1"/>
-        <v>299</v>
+        <v>329</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="17" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C21" s="12">
         <v>31.0</v>
@@ -2886,18 +2940,20 @@
       <c r="T21" s="13"/>
       <c r="U21" s="15"/>
       <c r="V21" s="14"/>
-      <c r="W21" s="15"/>
+      <c r="W21" s="12">
+        <v>26.0</v>
+      </c>
       <c r="X21" s="14"/>
       <c r="Y21" s="15"/>
       <c r="Z21" s="18"/>
       <c r="AA21" s="14">
         <f t="shared" si="1"/>
-        <v>160</v>
+        <v>186</v>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="28" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C22" s="12"/>
       <c r="D22" s="13"/>
@@ -2968,69 +3024,71 @@
     </row>
     <row r="24" ht="84.75" customHeight="1">
       <c r="B24" s="23" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C24" s="24" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D24" s="24" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E24" s="24" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F24" s="24" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G24" s="24" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H24" s="24" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I24" s="24" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="J24" s="24" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="K24" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="L24" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="M24" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="N24" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="O24" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="P24" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q24" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="R24" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="L24" s="24" t="s">
-        <v>96</v>
-      </c>
-      <c r="M24" s="24" t="s">
-        <v>84</v>
-      </c>
-      <c r="N24" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="O24" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="P24" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="Q24" s="24" t="s">
-        <v>96</v>
-      </c>
-      <c r="R24" s="24" t="s">
-        <v>89</v>
-      </c>
       <c r="S24" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="T24" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="U24" s="24" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="V24" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="W24" s="24"/>
+        <v>62</v>
+      </c>
+      <c r="W24" s="24" t="s">
+        <v>86</v>
+      </c>
       <c r="X24" s="24"/>
       <c r="Y24" s="24"/>
       <c r="Z24" s="24"/>
@@ -3038,7 +3096,7 @@
     </row>
     <row r="25">
       <c r="B25" s="26" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C25" s="27">
         <v>38.0</v>
@@ -3088,7 +3146,9 @@
         <v>36.0</v>
       </c>
       <c r="V25" s="27"/>
-      <c r="W25" s="27"/>
+      <c r="W25" s="27">
+        <v>38.0</v>
+      </c>
       <c r="X25" s="27"/>
       <c r="Y25" s="27"/>
       <c r="Z25" s="27"/>
@@ -3113,18 +3173,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="30" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B1" s="31" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C1" s="32" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="11" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B2" s="33"/>
       <c r="C2" s="34">
@@ -3133,16 +3193,16 @@
     </row>
     <row r="3">
       <c r="A3" s="17" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B3" s="33"/>
       <c r="C3" s="34">
-        <v>6.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="17" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B4" s="33"/>
       <c r="C4" s="34">
@@ -3151,7 +3211,7 @@
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B5" s="33"/>
       <c r="C5" s="34">
@@ -3160,7 +3220,7 @@
     </row>
     <row r="6">
       <c r="A6" s="17" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B6" s="33"/>
       <c r="C6" s="34">
@@ -3169,25 +3229,25 @@
     </row>
     <row r="7">
       <c r="A7" s="17" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B7" s="33"/>
       <c r="C7" s="34">
-        <v>10.0</v>
+        <v>11.0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="17" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B8" s="33"/>
       <c r="C8" s="34">
-        <v>14.0</v>
+        <v>13.0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="17" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B9" s="33"/>
       <c r="C9" s="34">
@@ -3196,7 +3256,7 @@
     </row>
     <row r="10">
       <c r="A10" s="17" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B10" s="33"/>
       <c r="C10" s="34">
@@ -3205,7 +3265,7 @@
     </row>
     <row r="11">
       <c r="A11" s="17" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B11" s="33"/>
       <c r="C11" s="34">
@@ -3214,7 +3274,7 @@
     </row>
     <row r="12">
       <c r="A12" s="17" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B12" s="33"/>
       <c r="C12" s="35">
@@ -3223,7 +3283,7 @@
     </row>
     <row r="13">
       <c r="A13" s="17" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B13" s="33"/>
       <c r="C13" s="34">
@@ -3232,7 +3292,7 @@
     </row>
     <row r="14">
       <c r="A14" s="17" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B14" s="33"/>
       <c r="C14" s="34">
@@ -3241,7 +3301,7 @@
     </row>
     <row r="15">
       <c r="A15" s="17" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B15" s="33"/>
       <c r="C15" s="34">
@@ -3250,7 +3310,7 @@
     </row>
     <row r="16">
       <c r="A16" s="17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B16" s="33"/>
       <c r="C16" s="34">
@@ -3259,7 +3319,7 @@
     </row>
     <row r="17">
       <c r="A17" s="17" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B17" s="33"/>
       <c r="C17" s="34">
@@ -3268,7 +3328,7 @@
     </row>
     <row r="18">
       <c r="A18" s="17" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B18" s="33"/>
       <c r="C18" s="34">
@@ -3277,7 +3337,7 @@
     </row>
     <row r="19">
       <c r="A19" s="17" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B19" s="33"/>
       <c r="C19" s="34">
@@ -3286,7 +3346,7 @@
     </row>
     <row r="20">
       <c r="A20" s="36" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B20" s="33"/>
       <c r="C20" s="34">
@@ -3295,34 +3355,34 @@
     </row>
     <row r="21">
       <c r="A21" s="17" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B21" s="33"/>
       <c r="C21" s="34">
-        <v>21.0</v>
+        <v>22.0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="17" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B22" s="33"/>
       <c r="C22" s="34">
-        <v>6.0</v>
+        <v>7.0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="17" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B23" s="33"/>
       <c r="C23" s="34">
-        <v>10.0</v>
+        <v>9.0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B24" s="37"/>
       <c r="C24" s="38">
@@ -3331,7 +3391,7 @@
     </row>
     <row r="25">
       <c r="A25" s="36" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B25" s="14"/>
       <c r="C25" s="13">
@@ -7241,13 +7301,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B1" s="39" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C1" s="40" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2">
@@ -7255,10 +7315,10 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="42" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C2" s="43" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3">
@@ -7266,10 +7326,10 @@
         <v>2.0</v>
       </c>
       <c r="B3" s="44" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C3" s="45" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4">
@@ -7277,10 +7337,10 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="44" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C4" s="45" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5">
@@ -7288,10 +7348,10 @@
         <v>4.0</v>
       </c>
       <c r="B5" s="44" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C5" s="45" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6">
@@ -7299,10 +7359,10 @@
         <v>5.0</v>
       </c>
       <c r="B6" s="44" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C6" s="45" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7">
@@ -7310,10 +7370,10 @@
         <v>6.0</v>
       </c>
       <c r="B7" s="44" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C7" s="45" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8">
@@ -7321,10 +7381,10 @@
         <v>7.0</v>
       </c>
       <c r="B8" s="44" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C8" s="45" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9">
@@ -7332,10 +7392,10 @@
         <v>8.0</v>
       </c>
       <c r="B9" s="44" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C9" s="45" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10">
@@ -7343,10 +7403,10 @@
         <v>9.0</v>
       </c>
       <c r="B10" s="44" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C10" s="45" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G10" s="14"/>
     </row>
@@ -7355,10 +7415,10 @@
         <v>10.0</v>
       </c>
       <c r="B11" s="44" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C11" s="45" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12">
@@ -7366,10 +7426,10 @@
         <v>11.0</v>
       </c>
       <c r="B12" s="44" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C12" s="45" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13">
@@ -7377,10 +7437,10 @@
         <v>12.0</v>
       </c>
       <c r="B13" s="44" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C13" s="45" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14">
@@ -7388,10 +7448,10 @@
         <v>13.0</v>
       </c>
       <c r="B14" s="44" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C14" s="45" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="15">
@@ -7399,10 +7459,10 @@
         <v>14.0</v>
       </c>
       <c r="B15" s="44" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C15" s="45" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16">
@@ -7410,10 +7470,10 @@
         <v>15.0</v>
       </c>
       <c r="B16" s="44" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C16" s="45" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17">
@@ -7421,10 +7481,10 @@
         <v>16.0</v>
       </c>
       <c r="B17" s="44" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C17" s="45" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18">
@@ -7432,10 +7492,10 @@
         <v>17.0</v>
       </c>
       <c r="B18" s="44" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C18" s="45" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19">
@@ -7443,10 +7503,10 @@
         <v>18.0</v>
       </c>
       <c r="B19" s="44" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C19" s="45" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="20">
@@ -7454,10 +7514,10 @@
         <v>19.0</v>
       </c>
       <c r="B20" s="44" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C20" s="45" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="21">
@@ -7465,18 +7525,22 @@
         <v>20.0</v>
       </c>
       <c r="B21" s="44" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C21" s="45" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="13">
         <v>21.0</v>
       </c>
-      <c r="B22" s="44"/>
-      <c r="C22" s="45"/>
+      <c r="B22" s="44" t="s">
+        <v>94</v>
+      </c>
+      <c r="C22" s="45" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="13">
@@ -12373,19 +12437,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D1" s="46" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E1" s="26" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2">
@@ -12814,19 +12878,19 @@
       </c>
       <c r="B22" s="47" t="str">
         <f>'SUNDAY SINGLES'!W24</f>
-        <v/>
-      </c>
-      <c r="C22" s="47" t="str">
+        <v>MICK SKINNER</v>
+      </c>
+      <c r="C22" s="47">
         <f>'SUNDAY SINGLES'!W25</f>
-        <v/>
+        <v>38</v>
       </c>
       <c r="D22" s="48" t="str">
         <f>'THURSDAY SINGLES'!W19</f>
-        <v/>
-      </c>
-      <c r="E22" s="47" t="str">
+        <v>ALBIE GILLESPIE</v>
+      </c>
+      <c r="E22" s="47">
         <f>'THURSDAY SINGLES'!W20</f>
-        <v/>
+        <v>41</v>
       </c>
     </row>
     <row r="23">

</xml_diff>

<commit_message>
089 Week 22/22 data update
</commit_message>
<xml_diff>
--- a/data/WINTER_GOLF_2526.xlsx
+++ b/data/WINTER_GOLF_2526.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="116">
   <si>
     <t>WINTER GOLF 25/26 - THURSDAY SINGLES</t>
   </si>
@@ -81,6 +81,15 @@
   </si>
   <si>
     <t>5th March 26</t>
+  </si>
+  <si>
+    <t>12th March 26</t>
+  </si>
+  <si>
+    <t>19th  March 26</t>
+  </si>
+  <si>
+    <t>26th March 26</t>
   </si>
   <si>
     <t>NAME</t>
@@ -275,6 +284,15 @@
     <t>8th March 26</t>
   </si>
   <si>
+    <t>15th  March 26</t>
+  </si>
+  <si>
+    <t>22nd March 26</t>
+  </si>
+  <si>
+    <t>29th March 26</t>
+  </si>
+  <si>
     <t>MICK SKINNER</t>
   </si>
   <si>
@@ -312,6 +330,9 @@
   </si>
   <si>
     <t>PAUL HANCOX</t>
+  </si>
+  <si>
+    <t>NATHAN DEAKIN</t>
   </si>
   <si>
     <t>WHITE TEES</t>
@@ -967,94 +988,100 @@
       <c r="W3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="X3" s="4"/>
-      <c r="Y3" s="3"/>
-      <c r="Z3" s="5"/>
+      <c r="X3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="Z3" s="5" t="s">
+        <v>24</v>
+      </c>
       <c r="AA3" s="6"/>
     </row>
     <row r="4">
       <c r="B4" s="7" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="Q4" s="8" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="R4" s="8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="S4" s="8" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="T4" s="8" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="U4" s="8" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="V4" s="8" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="W4" s="8" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="X4" s="8" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="Y4" s="8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="Z4" s="8" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AA4" s="10" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="11" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="13">
@@ -1111,7 +1138,7 @@
     </row>
     <row r="6">
       <c r="B6" s="17" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C6" s="12">
         <v>28.0</v>
@@ -1158,17 +1185,19 @@
       <c r="W6" s="12">
         <v>35.0</v>
       </c>
-      <c r="X6" s="13"/>
+      <c r="X6" s="13">
+        <v>30.0</v>
+      </c>
       <c r="Y6" s="12"/>
       <c r="Z6" s="18"/>
       <c r="AA6" s="14">
         <f t="shared" si="1"/>
-        <v>353</v>
+        <v>383</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="17" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C7" s="12">
         <v>31.0</v>
@@ -1213,17 +1242,19 @@
       <c r="W7" s="12">
         <v>36.0</v>
       </c>
-      <c r="X7" s="14"/>
+      <c r="X7" s="13">
+        <v>29.0</v>
+      </c>
       <c r="Y7" s="12"/>
       <c r="Z7" s="18"/>
       <c r="AA7" s="14">
         <f t="shared" si="1"/>
-        <v>375</v>
+        <v>404</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="17" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C8" s="12">
         <v>31.0</v>
@@ -1264,17 +1295,19 @@
       <c r="W8" s="12">
         <v>32.0</v>
       </c>
-      <c r="X8" s="13"/>
+      <c r="X8" s="13">
+        <v>34.0</v>
+      </c>
       <c r="Y8" s="12"/>
       <c r="Z8" s="16"/>
       <c r="AA8" s="14">
         <f t="shared" si="1"/>
-        <v>300</v>
+        <v>334</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="17" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C9" s="12">
         <v>34.0</v>
@@ -1331,7 +1364,7 @@
     </row>
     <row r="10">
       <c r="B10" s="17" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C10" s="12">
         <v>21.0</v>
@@ -1366,17 +1399,19 @@
         <v>41.0</v>
       </c>
       <c r="W10" s="12"/>
-      <c r="X10" s="13"/>
+      <c r="X10" s="13">
+        <v>30.0</v>
+      </c>
       <c r="Y10" s="12"/>
       <c r="Z10" s="16"/>
       <c r="AA10" s="14">
         <f t="shared" si="1"/>
-        <v>196</v>
+        <v>226</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="17" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C11" s="12">
         <v>36.0</v>
@@ -1423,17 +1458,19 @@
       <c r="W11" s="12">
         <v>30.0</v>
       </c>
-      <c r="X11" s="13"/>
+      <c r="X11" s="13">
+        <v>35.0</v>
+      </c>
       <c r="Y11" s="12"/>
       <c r="Z11" s="16"/>
       <c r="AA11" s="14">
         <f t="shared" si="1"/>
-        <v>334</v>
+        <v>369</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="17" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C12" s="12">
         <v>35.0</v>
@@ -1486,7 +1523,7 @@
     </row>
     <row r="13">
       <c r="B13" s="17" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C13" s="12">
         <v>34.0</v>
@@ -1533,7 +1570,7 @@
     </row>
     <row r="14">
       <c r="B14" s="17" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C14" s="12">
         <v>33.0</v>
@@ -1586,17 +1623,19 @@
       <c r="W14" s="12">
         <v>41.0</v>
       </c>
-      <c r="X14" s="13"/>
+      <c r="X14" s="13">
+        <v>34.0</v>
+      </c>
       <c r="Y14" s="12"/>
       <c r="Z14" s="18"/>
       <c r="AA14" s="14">
         <f t="shared" si="1"/>
-        <v>494</v>
+        <v>528</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="17" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="13"/>
@@ -1647,17 +1686,19 @@
       <c r="W15" s="12">
         <v>30.0</v>
       </c>
-      <c r="X15" s="13"/>
+      <c r="X15" s="13">
+        <v>26.0</v>
+      </c>
       <c r="Y15" s="12"/>
       <c r="Z15" s="18"/>
       <c r="AA15" s="14">
         <f t="shared" si="1"/>
-        <v>428</v>
+        <v>454</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="19" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C16" s="18">
         <v>26.0</v>
@@ -1708,7 +1749,7 @@
     </row>
     <row r="17">
       <c r="B17" s="21" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C17" s="12">
         <v>31.0</v>
@@ -1787,79 +1828,81 @@
     </row>
     <row r="19" ht="72.0" customHeight="1">
       <c r="B19" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="C19" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="D19" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="E19" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="F19" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="G19" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="C19" s="24" t="s">
-        <v>54</v>
-      </c>
-      <c r="D19" s="24" t="s">
-        <v>50</v>
-      </c>
-      <c r="E19" s="24" t="s">
+      <c r="H19" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="I19" s="24" t="s">
         <v>51</v>
       </c>
-      <c r="F19" s="24" t="s">
-        <v>52</v>
-      </c>
-      <c r="G19" s="24" t="s">
+      <c r="J19" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="H19" s="24" t="s">
-        <v>50</v>
-      </c>
-      <c r="I19" s="24" t="s">
-        <v>48</v>
-      </c>
-      <c r="J19" s="24" t="s">
-        <v>55</v>
-      </c>
       <c r="K19" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="L19" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="M19" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="N19" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="O19" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="P19" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q19" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="R19" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="S19" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="T19" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="U19" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="V19" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="W19" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="X19" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="L19" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="M19" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="N19" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="O19" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="P19" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q19" s="24" t="s">
-        <v>57</v>
-      </c>
-      <c r="R19" s="24" t="s">
-        <v>57</v>
-      </c>
-      <c r="S19" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="T19" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="U19" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="V19" s="24" t="s">
-        <v>53</v>
-      </c>
-      <c r="W19" s="24" t="s">
-        <v>57</v>
-      </c>
-      <c r="X19" s="24"/>
       <c r="Y19" s="24"/>
       <c r="Z19" s="24"/>
       <c r="AA19" s="25"/>
     </row>
     <row r="20">
       <c r="B20" s="26" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C20" s="27">
         <v>36.0</v>
@@ -1914,7 +1957,9 @@
       <c r="W20" s="27">
         <v>41.0</v>
       </c>
-      <c r="X20" s="27"/>
+      <c r="X20" s="27">
+        <v>35.0</v>
+      </c>
       <c r="Y20" s="27"/>
       <c r="Z20" s="27"/>
     </row>
@@ -1938,163 +1983,169 @@
   <sheetData>
     <row r="2" ht="24.0" customHeight="1">
       <c r="B2" s="1" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="Z2" s="2"/>
       <c r="AA2" s="2"/>
     </row>
     <row r="3" ht="73.5" customHeight="1">
       <c r="C3" s="3" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="R3" s="4" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="S3" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="T3" s="4" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="U3" s="3" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="V3" s="4" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="W3" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="X3" s="4"/>
-      <c r="Y3" s="3"/>
-      <c r="Z3" s="5"/>
+        <v>88</v>
+      </c>
+      <c r="X3" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y3" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z3" s="5" t="s">
+        <v>91</v>
+      </c>
       <c r="AA3" s="6"/>
     </row>
     <row r="4">
       <c r="B4" s="7" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="Q4" s="8" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="R4" s="8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="S4" s="8" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="T4" s="8" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="U4" s="8" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="V4" s="8" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="W4" s="8" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="X4" s="8" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="Y4" s="8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="Z4" s="8" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AA4" s="10" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="11" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="13"/>
@@ -2131,7 +2182,7 @@
     </row>
     <row r="6">
       <c r="B6" s="17" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="C6" s="12">
         <v>38.0</v>
@@ -2168,17 +2219,19 @@
       <c r="W6" s="12">
         <v>38.0</v>
       </c>
-      <c r="X6" s="13"/>
+      <c r="X6" s="13">
+        <v>34.0</v>
+      </c>
       <c r="Y6" s="12"/>
       <c r="Z6" s="16"/>
       <c r="AA6" s="14">
         <f t="shared" si="1"/>
-        <v>259</v>
+        <v>293</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="17" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="13">
@@ -2237,7 +2290,7 @@
     </row>
     <row r="8">
       <c r="B8" s="17" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C8" s="12">
         <v>28.0</v>
@@ -2286,7 +2339,7 @@
     </row>
     <row r="9">
       <c r="B9" s="17" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="13">
@@ -2323,17 +2376,19 @@
       <c r="W9" s="12">
         <v>34.0</v>
       </c>
-      <c r="X9" s="13"/>
+      <c r="X9" s="13">
+        <v>35.0</v>
+      </c>
       <c r="Y9" s="15"/>
       <c r="Z9" s="16"/>
       <c r="AA9" s="14">
         <f t="shared" si="1"/>
-        <v>232</v>
+        <v>267</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="17" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C10" s="15"/>
       <c r="D10" s="13"/>
@@ -2380,7 +2435,7 @@
     </row>
     <row r="11">
       <c r="B11" s="17" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="C11" s="12">
         <v>33.0</v>
@@ -2415,17 +2470,19 @@
       <c r="U11" s="15"/>
       <c r="V11" s="14"/>
       <c r="W11" s="12"/>
-      <c r="X11" s="13"/>
+      <c r="X11" s="13">
+        <v>33.0</v>
+      </c>
       <c r="Y11" s="12"/>
       <c r="Z11" s="16"/>
       <c r="AA11" s="14">
         <f t="shared" si="1"/>
-        <v>210</v>
+        <v>243</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="17" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="13"/>
@@ -2468,7 +2525,7 @@
     </row>
     <row r="13">
       <c r="B13" s="17" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="C13" s="12">
         <v>33.0</v>
@@ -2521,7 +2578,7 @@
     </row>
     <row r="14">
       <c r="B14" s="17" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C14" s="12">
         <v>29.0</v>
@@ -2578,7 +2635,7 @@
     </row>
     <row r="15">
       <c r="B15" s="17" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C15" s="12">
         <v>28.0</v>
@@ -2623,17 +2680,19 @@
       </c>
       <c r="V15" s="13"/>
       <c r="W15" s="12"/>
-      <c r="X15" s="13"/>
+      <c r="X15" s="13">
+        <v>32.0</v>
+      </c>
       <c r="Y15" s="12"/>
       <c r="Z15" s="16"/>
       <c r="AA15" s="14">
         <f t="shared" si="1"/>
-        <v>320</v>
+        <v>352</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="17" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C16" s="12">
         <v>24.0</v>
@@ -2676,17 +2735,19 @@
       <c r="W16" s="12">
         <v>27.0</v>
       </c>
-      <c r="X16" s="13"/>
+      <c r="X16" s="13">
+        <v>26.0</v>
+      </c>
       <c r="Y16" s="12"/>
       <c r="Z16" s="16"/>
       <c r="AA16" s="14">
         <f t="shared" si="1"/>
-        <v>301</v>
+        <v>327</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="17" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C17" s="12">
         <v>31.0</v>
@@ -2743,7 +2804,7 @@
     </row>
     <row r="18">
       <c r="B18" s="17" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C18" s="12">
         <v>35.0</v>
@@ -2780,17 +2841,19 @@
       <c r="W18" s="12">
         <v>37.0</v>
       </c>
-      <c r="X18" s="13"/>
+      <c r="X18" s="13">
+        <v>35.0</v>
+      </c>
       <c r="Y18" s="12"/>
       <c r="Z18" s="18"/>
       <c r="AA18" s="14">
         <f t="shared" si="1"/>
-        <v>233</v>
+        <v>268</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="17" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="C19" s="12">
         <v>33.0</v>
@@ -2841,17 +2904,19 @@
       <c r="W19" s="12">
         <v>32.0</v>
       </c>
-      <c r="X19" s="13"/>
+      <c r="X19" s="13">
+        <v>31.0</v>
+      </c>
       <c r="Y19" s="12"/>
       <c r="Z19" s="16"/>
       <c r="AA19" s="14">
         <f t="shared" si="1"/>
-        <v>453</v>
+        <v>484</v>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="17" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="C20" s="12">
         <v>27.0</v>
@@ -2896,17 +2961,19 @@
       <c r="W20" s="12">
         <v>30.0</v>
       </c>
-      <c r="X20" s="14"/>
+      <c r="X20" s="13">
+        <v>27.0</v>
+      </c>
       <c r="Y20" s="12"/>
       <c r="Z20" s="18"/>
       <c r="AA20" s="14">
         <f t="shared" si="1"/>
-        <v>329</v>
+        <v>356</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="17" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="C21" s="12">
         <v>31.0</v>
@@ -2953,7 +3020,7 @@
     </row>
     <row r="22">
       <c r="B22" s="28" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C22" s="12"/>
       <c r="D22" s="13"/>
@@ -3024,79 +3091,81 @@
     </row>
     <row r="24" ht="84.75" customHeight="1">
       <c r="B24" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="C24" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="D24" s="24" t="s">
+        <v>97</v>
+      </c>
+      <c r="E24" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="F24" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="G24" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="C24" s="24" t="s">
-        <v>86</v>
-      </c>
-      <c r="D24" s="24" t="s">
-        <v>91</v>
-      </c>
-      <c r="E24" s="24" t="s">
-        <v>87</v>
-      </c>
-      <c r="F24" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="G24" s="24" t="s">
-        <v>58</v>
-      </c>
       <c r="H24" s="24" t="s">
+        <v>102</v>
+      </c>
+      <c r="I24" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="J24" s="24" t="s">
+        <v>103</v>
+      </c>
+      <c r="K24" s="24" t="s">
+        <v>99</v>
+      </c>
+      <c r="L24" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="M24" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="N24" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="O24" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="P24" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q24" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="R24" s="24" t="s">
+        <v>97</v>
+      </c>
+      <c r="S24" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="T24" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="U24" s="24" t="s">
         <v>96</v>
       </c>
-      <c r="I24" s="24" t="s">
-        <v>86</v>
-      </c>
-      <c r="J24" s="24" t="s">
-        <v>97</v>
-      </c>
-      <c r="K24" s="24" t="s">
-        <v>93</v>
-      </c>
-      <c r="L24" s="24" t="s">
-        <v>98</v>
-      </c>
-      <c r="M24" s="24" t="s">
-        <v>86</v>
-      </c>
-      <c r="N24" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="O24" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="P24" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="Q24" s="24" t="s">
-        <v>98</v>
-      </c>
-      <c r="R24" s="24" t="s">
-        <v>91</v>
-      </c>
-      <c r="S24" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="T24" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="U24" s="24" t="s">
-        <v>90</v>
-      </c>
       <c r="V24" s="24" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="W24" s="24" t="s">
-        <v>86</v>
-      </c>
-      <c r="X24" s="24"/>
+        <v>92</v>
+      </c>
+      <c r="X24" s="24" t="s">
+        <v>105</v>
+      </c>
       <c r="Y24" s="24"/>
       <c r="Z24" s="24"/>
       <c r="AA24" s="29"/>
     </row>
     <row r="25">
       <c r="B25" s="26" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C25" s="27">
         <v>38.0</v>
@@ -3149,7 +3218,9 @@
       <c r="W25" s="27">
         <v>38.0</v>
       </c>
-      <c r="X25" s="27"/>
+      <c r="X25" s="27">
+        <v>36.0</v>
+      </c>
       <c r="Y25" s="27"/>
       <c r="Z25" s="27"/>
       <c r="AA25" s="14"/>
@@ -3173,18 +3244,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="30" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B1" s="31" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="C1" s="32" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="11" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="B2" s="33"/>
       <c r="C2" s="34">
@@ -3193,7 +3264,7 @@
     </row>
     <row r="3">
       <c r="A3" s="17" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B3" s="33"/>
       <c r="C3" s="34">
@@ -3202,7 +3273,7 @@
     </row>
     <row r="4">
       <c r="A4" s="17" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="B4" s="33"/>
       <c r="C4" s="34">
@@ -3211,7 +3282,7 @@
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="B5" s="33"/>
       <c r="C5" s="34">
@@ -3220,7 +3291,7 @@
     </row>
     <row r="6">
       <c r="A6" s="17" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="B6" s="33"/>
       <c r="C6" s="34">
@@ -3229,7 +3300,7 @@
     </row>
     <row r="7">
       <c r="A7" s="17" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="B7" s="33"/>
       <c r="C7" s="34">
@@ -3238,7 +3309,7 @@
     </row>
     <row r="8">
       <c r="A8" s="17" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B8" s="33"/>
       <c r="C8" s="34">
@@ -3247,7 +3318,7 @@
     </row>
     <row r="9">
       <c r="A9" s="17" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B9" s="33"/>
       <c r="C9" s="34">
@@ -3256,7 +3327,7 @@
     </row>
     <row r="10">
       <c r="A10" s="17" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="B10" s="33"/>
       <c r="C10" s="34">
@@ -3265,7 +3336,7 @@
     </row>
     <row r="11">
       <c r="A11" s="17" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B11" s="33"/>
       <c r="C11" s="34">
@@ -3274,7 +3345,7 @@
     </row>
     <row r="12">
       <c r="A12" s="17" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B12" s="33"/>
       <c r="C12" s="35">
@@ -3283,7 +3354,7 @@
     </row>
     <row r="13">
       <c r="A13" s="17" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B13" s="33"/>
       <c r="C13" s="34">
@@ -3292,7 +3363,7 @@
     </row>
     <row r="14">
       <c r="A14" s="17" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B14" s="33"/>
       <c r="C14" s="34">
@@ -3301,7 +3372,7 @@
     </row>
     <row r="15">
       <c r="A15" s="17" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B15" s="33"/>
       <c r="C15" s="34">
@@ -3310,7 +3381,7 @@
     </row>
     <row r="16">
       <c r="A16" s="17" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B16" s="33"/>
       <c r="C16" s="34">
@@ -3319,7 +3390,7 @@
     </row>
     <row r="17">
       <c r="A17" s="17" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B17" s="33"/>
       <c r="C17" s="34">
@@ -3328,7 +3399,7 @@
     </row>
     <row r="18">
       <c r="A18" s="17" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="B18" s="33"/>
       <c r="C18" s="34">
@@ -3337,7 +3408,7 @@
     </row>
     <row r="19">
       <c r="A19" s="17" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="B19" s="33"/>
       <c r="C19" s="34">
@@ -3346,7 +3417,7 @@
     </row>
     <row r="20">
       <c r="A20" s="36" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B20" s="33"/>
       <c r="C20" s="34">
@@ -3355,7 +3426,7 @@
     </row>
     <row r="21">
       <c r="A21" s="17" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="B21" s="33"/>
       <c r="C21" s="34">
@@ -3364,7 +3435,7 @@
     </row>
     <row r="22">
       <c r="A22" s="17" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B22" s="33"/>
       <c r="C22" s="34">
@@ -3373,7 +3444,7 @@
     </row>
     <row r="23">
       <c r="A23" s="17" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B23" s="33"/>
       <c r="C23" s="34">
@@ -3382,7 +3453,7 @@
     </row>
     <row r="24">
       <c r="A24" s="28" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="B24" s="37"/>
       <c r="C24" s="38">
@@ -3391,7 +3462,7 @@
     </row>
     <row r="25">
       <c r="A25" s="36" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B25" s="14"/>
       <c r="C25" s="13">
@@ -7301,13 +7372,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="B1" s="39" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="C1" s="40" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2">
@@ -7315,10 +7386,10 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="42" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="C2" s="43" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3">
@@ -7326,10 +7397,10 @@
         <v>2.0</v>
       </c>
       <c r="B3" s="44" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C3" s="45" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4">
@@ -7337,10 +7408,10 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="44" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="C4" s="45" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5">
@@ -7348,10 +7419,10 @@
         <v>4.0</v>
       </c>
       <c r="B5" s="44" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C5" s="45" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6">
@@ -7359,10 +7430,10 @@
         <v>5.0</v>
       </c>
       <c r="B6" s="44" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C6" s="45" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7">
@@ -7370,10 +7441,10 @@
         <v>6.0</v>
       </c>
       <c r="B7" s="44" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C7" s="45" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8">
@@ -7381,10 +7452,10 @@
         <v>7.0</v>
       </c>
       <c r="B8" s="44" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="45" t="s">
         <v>62</v>
-      </c>
-      <c r="C8" s="45" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="9">
@@ -7392,10 +7463,10 @@
         <v>8.0</v>
       </c>
       <c r="B9" s="44" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C9" s="45" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10">
@@ -7403,10 +7474,10 @@
         <v>9.0</v>
       </c>
       <c r="B10" s="44" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C10" s="45" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="G10" s="14"/>
     </row>
@@ -7415,10 +7486,10 @@
         <v>10.0</v>
       </c>
       <c r="B11" s="44" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="C11" s="45" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12">
@@ -7426,10 +7497,10 @@
         <v>11.0</v>
       </c>
       <c r="B12" s="44" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C12" s="45" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13">
@@ -7437,10 +7508,10 @@
         <v>12.0</v>
       </c>
       <c r="B13" s="44" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C13" s="45" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14">
@@ -7448,10 +7519,10 @@
         <v>13.0</v>
       </c>
       <c r="B14" s="44" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C14" s="45" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="15">
@@ -7459,10 +7530,10 @@
         <v>14.0</v>
       </c>
       <c r="B15" s="44" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C15" s="45" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="16">
@@ -7470,10 +7541,10 @@
         <v>15.0</v>
       </c>
       <c r="B16" s="44" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C16" s="45" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="17">
@@ -7481,10 +7552,10 @@
         <v>16.0</v>
       </c>
       <c r="B17" s="44" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C17" s="45" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18">
@@ -7492,10 +7563,10 @@
         <v>17.0</v>
       </c>
       <c r="B18" s="44" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C18" s="45" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="19">
@@ -7503,10 +7574,10 @@
         <v>18.0</v>
       </c>
       <c r="B19" s="44" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C19" s="45" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="20">
@@ -7514,10 +7585,10 @@
         <v>19.0</v>
       </c>
       <c r="B20" s="44" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="C20" s="45" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="21">
@@ -7525,10 +7596,10 @@
         <v>20.0</v>
       </c>
       <c r="B21" s="44" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C21" s="45" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22">
@@ -7536,18 +7607,22 @@
         <v>21.0</v>
       </c>
       <c r="B22" s="44" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="C22" s="45" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="13">
         <v>22.0</v>
       </c>
-      <c r="B23" s="44"/>
-      <c r="C23" s="45"/>
+      <c r="B23" s="44" t="s">
+        <v>93</v>
+      </c>
+      <c r="C23" s="45" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="13">
@@ -12437,19 +12512,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="D1" s="46" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="E1" s="26" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2">
@@ -12899,19 +12974,19 @@
       </c>
       <c r="B23" s="47" t="str">
         <f>'SUNDAY SINGLES'!X24</f>
-        <v/>
-      </c>
-      <c r="C23" s="47" t="str">
+        <v>NATHAN DEAKIN</v>
+      </c>
+      <c r="C23" s="47">
         <f>'SUNDAY SINGLES'!X25</f>
-        <v/>
+        <v>36</v>
       </c>
       <c r="D23" s="48" t="str">
         <f>'THURSDAY SINGLES'!X19</f>
-        <v/>
-      </c>
-      <c r="E23" s="47" t="str">
+        <v>JOHN ANTCLIFFE</v>
+      </c>
+      <c r="E23" s="47">
         <f>'THURSDAY SINGLES'!X20</f>
-        <v/>
+        <v>35</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
090 Week 23/23 data update
</commit_message>
<xml_diff>
--- a/data/WINTER_GOLF_2526.xlsx
+++ b/data/WINTER_GOLF_2526.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="116">
   <si>
     <t>WINTER GOLF 25/26 - THURSDAY SINGLES</t>
   </si>
@@ -1188,11 +1188,13 @@
       <c r="X6" s="13">
         <v>30.0</v>
       </c>
-      <c r="Y6" s="12"/>
+      <c r="Y6" s="12">
+        <v>28.0</v>
+      </c>
       <c r="Z6" s="18"/>
       <c r="AA6" s="14">
         <f t="shared" si="1"/>
-        <v>383</v>
+        <v>411</v>
       </c>
     </row>
     <row r="7">
@@ -1245,11 +1247,13 @@
       <c r="X7" s="13">
         <v>29.0</v>
       </c>
-      <c r="Y7" s="12"/>
+      <c r="Y7" s="12">
+        <v>31.0</v>
+      </c>
       <c r="Z7" s="18"/>
       <c r="AA7" s="14">
         <f t="shared" si="1"/>
-        <v>404</v>
+        <v>435</v>
       </c>
     </row>
     <row r="8">
@@ -1298,11 +1302,13 @@
       <c r="X8" s="13">
         <v>34.0</v>
       </c>
-      <c r="Y8" s="12"/>
+      <c r="Y8" s="12">
+        <v>25.0</v>
+      </c>
       <c r="Z8" s="16"/>
       <c r="AA8" s="14">
         <f t="shared" si="1"/>
-        <v>334</v>
+        <v>359</v>
       </c>
     </row>
     <row r="9">
@@ -1355,11 +1361,13 @@
         <v>28.0</v>
       </c>
       <c r="X9" s="14"/>
-      <c r="Y9" s="15"/>
+      <c r="Y9" s="12">
+        <v>24.0</v>
+      </c>
       <c r="Z9" s="16"/>
       <c r="AA9" s="14">
         <f t="shared" si="1"/>
-        <v>360</v>
+        <v>384</v>
       </c>
     </row>
     <row r="10">
@@ -1402,11 +1410,13 @@
       <c r="X10" s="13">
         <v>30.0</v>
       </c>
-      <c r="Y10" s="12"/>
+      <c r="Y10" s="12">
+        <v>23.0</v>
+      </c>
       <c r="Z10" s="16"/>
       <c r="AA10" s="14">
         <f t="shared" si="1"/>
-        <v>226</v>
+        <v>249</v>
       </c>
     </row>
     <row r="11">
@@ -1896,7 +1906,9 @@
       <c r="X19" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="Y19" s="24"/>
+      <c r="Y19" s="24" t="s">
+        <v>53</v>
+      </c>
       <c r="Z19" s="24"/>
       <c r="AA19" s="25"/>
     </row>
@@ -1960,7 +1972,9 @@
       <c r="X20" s="27">
         <v>35.0</v>
       </c>
-      <c r="Y20" s="27"/>
+      <c r="Y20" s="27">
+        <v>31.0</v>
+      </c>
       <c r="Z20" s="27"/>
     </row>
   </sheetData>
@@ -2222,11 +2236,13 @@
       <c r="X6" s="13">
         <v>34.0</v>
       </c>
-      <c r="Y6" s="12"/>
+      <c r="Y6" s="12">
+        <v>30.0</v>
+      </c>
       <c r="Z6" s="16"/>
       <c r="AA6" s="14">
         <f t="shared" si="1"/>
-        <v>293</v>
+        <v>323</v>
       </c>
     </row>
     <row r="7">
@@ -2473,11 +2489,13 @@
       <c r="X11" s="13">
         <v>33.0</v>
       </c>
-      <c r="Y11" s="12"/>
+      <c r="Y11" s="12">
+        <v>33.0</v>
+      </c>
       <c r="Z11" s="16"/>
       <c r="AA11" s="14">
         <f t="shared" si="1"/>
-        <v>243</v>
+        <v>276</v>
       </c>
     </row>
     <row r="12">
@@ -2516,11 +2534,13 @@
       <c r="V12" s="14"/>
       <c r="W12" s="12"/>
       <c r="X12" s="13"/>
-      <c r="Y12" s="12"/>
+      <c r="Y12" s="12">
+        <v>31.0</v>
+      </c>
       <c r="Z12" s="18"/>
       <c r="AA12" s="14">
         <f t="shared" si="1"/>
-        <v>166</v>
+        <v>197</v>
       </c>
     </row>
     <row r="13">
@@ -2626,11 +2646,13 @@
       <c r="V14" s="13"/>
       <c r="W14" s="12"/>
       <c r="X14" s="13"/>
-      <c r="Y14" s="15"/>
+      <c r="Y14" s="12">
+        <v>30.0</v>
+      </c>
       <c r="Z14" s="16"/>
       <c r="AA14" s="14">
         <f t="shared" si="1"/>
-        <v>356</v>
+        <v>386</v>
       </c>
     </row>
     <row r="15">
@@ -2683,11 +2705,13 @@
       <c r="X15" s="13">
         <v>32.0</v>
       </c>
-      <c r="Y15" s="12"/>
+      <c r="Y15" s="12">
+        <v>36.0</v>
+      </c>
       <c r="Z15" s="16"/>
       <c r="AA15" s="14">
         <f t="shared" si="1"/>
-        <v>352</v>
+        <v>388</v>
       </c>
     </row>
     <row r="16">
@@ -2844,11 +2868,13 @@
       <c r="X18" s="13">
         <v>35.0</v>
       </c>
-      <c r="Y18" s="12"/>
+      <c r="Y18" s="12">
+        <v>38.0</v>
+      </c>
       <c r="Z18" s="18"/>
       <c r="AA18" s="14">
         <f t="shared" si="1"/>
-        <v>268</v>
+        <v>306</v>
       </c>
     </row>
     <row r="19">
@@ -2907,11 +2933,13 @@
       <c r="X19" s="13">
         <v>31.0</v>
       </c>
-      <c r="Y19" s="12"/>
+      <c r="Y19" s="12">
+        <v>38.0</v>
+      </c>
       <c r="Z19" s="16"/>
       <c r="AA19" s="14">
         <f t="shared" si="1"/>
-        <v>484</v>
+        <v>522</v>
       </c>
     </row>
     <row r="20">
@@ -2964,11 +2992,13 @@
       <c r="X20" s="13">
         <v>27.0</v>
       </c>
-      <c r="Y20" s="12"/>
+      <c r="Y20" s="12">
+        <v>31.0</v>
+      </c>
       <c r="Z20" s="18"/>
       <c r="AA20" s="14">
         <f t="shared" si="1"/>
-        <v>356</v>
+        <v>387</v>
       </c>
     </row>
     <row r="21">
@@ -3159,7 +3189,9 @@
       <c r="X24" s="24" t="s">
         <v>105</v>
       </c>
-      <c r="Y24" s="24"/>
+      <c r="Y24" s="24" t="s">
+        <v>99</v>
+      </c>
       <c r="Z24" s="24"/>
       <c r="AA24" s="29"/>
     </row>
@@ -3221,7 +3253,9 @@
       <c r="X25" s="27">
         <v>36.0</v>
       </c>
-      <c r="Y25" s="27"/>
+      <c r="Y25" s="27">
+        <v>38.0</v>
+      </c>
       <c r="Z25" s="27"/>
       <c r="AA25" s="14"/>
     </row>
@@ -3322,7 +3356,7 @@
       </c>
       <c r="B9" s="33"/>
       <c r="C9" s="34">
-        <v>10.0</v>
+        <v>11.0</v>
       </c>
     </row>
     <row r="10">
@@ -3385,7 +3419,7 @@
       </c>
       <c r="B16" s="33"/>
       <c r="C16" s="34">
-        <v>11.0</v>
+        <v>12.0</v>
       </c>
     </row>
     <row r="17">
@@ -7628,8 +7662,12 @@
       <c r="A24" s="13">
         <v>23.0</v>
       </c>
-      <c r="B24" s="44"/>
-      <c r="C24" s="45"/>
+      <c r="B24" s="44" t="s">
+        <v>98</v>
+      </c>
+      <c r="C24" s="45" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="13">
@@ -12995,19 +13033,19 @@
       </c>
       <c r="B24" s="47" t="str">
         <f>'SUNDAY SINGLES'!Y24</f>
-        <v/>
-      </c>
-      <c r="C24" s="47" t="str">
+        <v>CHRIS HARVEY</v>
+      </c>
+      <c r="C24" s="47">
         <f>'SUNDAY SINGLES'!Y25</f>
-        <v/>
+        <v>38</v>
       </c>
       <c r="D24" s="48" t="str">
         <f>'THURSDAY SINGLES'!Y19</f>
-        <v/>
-      </c>
-      <c r="E24" s="47" t="str">
+        <v>MARTIN BROCK</v>
+      </c>
+      <c r="E24" s="47">
         <f>'THURSDAY SINGLES'!Y20</f>
-        <v/>
+        <v>31</v>
       </c>
     </row>
     <row r="25">

</xml_diff>

<commit_message>
091 Final week data update
</commit_message>
<xml_diff>
--- a/data/WINTER_GOLF_2526.xlsx
+++ b/data/WINTER_GOLF_2526.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="116">
   <si>
     <t>WINTER GOLF 25/26 - THURSDAY SINGLES</t>
   </si>
@@ -590,13 +590,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="8" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="9" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="8" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="7" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -1130,10 +1130,12 @@
       </c>
       <c r="X5" s="14"/>
       <c r="Y5" s="15"/>
-      <c r="Z5" s="16"/>
+      <c r="Z5" s="16">
+        <v>25.0</v>
+      </c>
       <c r="AA5" s="14">
         <f t="shared" ref="AA5:AA17" si="1">sum(C5:Z5)</f>
-        <v>371</v>
+        <v>396</v>
       </c>
     </row>
     <row r="6">
@@ -1191,10 +1193,12 @@
       <c r="Y6" s="12">
         <v>28.0</v>
       </c>
-      <c r="Z6" s="18"/>
+      <c r="Z6" s="16">
+        <v>35.0</v>
+      </c>
       <c r="AA6" s="14">
         <f t="shared" si="1"/>
-        <v>411</v>
+        <v>446</v>
       </c>
     </row>
     <row r="7">
@@ -1250,7 +1254,7 @@
       <c r="Y7" s="12">
         <v>31.0</v>
       </c>
-      <c r="Z7" s="18"/>
+      <c r="Z7" s="16"/>
       <c r="AA7" s="14">
         <f t="shared" si="1"/>
         <v>435</v>
@@ -1305,7 +1309,7 @@
       <c r="Y8" s="12">
         <v>25.0</v>
       </c>
-      <c r="Z8" s="16"/>
+      <c r="Z8" s="18"/>
       <c r="AA8" s="14">
         <f t="shared" si="1"/>
         <v>359</v>
@@ -1364,10 +1368,12 @@
       <c r="Y9" s="12">
         <v>24.0</v>
       </c>
-      <c r="Z9" s="16"/>
+      <c r="Z9" s="16">
+        <v>26.0</v>
+      </c>
       <c r="AA9" s="14">
         <f t="shared" si="1"/>
-        <v>384</v>
+        <v>410</v>
       </c>
     </row>
     <row r="10">
@@ -1413,10 +1419,12 @@
       <c r="Y10" s="12">
         <v>23.0</v>
       </c>
-      <c r="Z10" s="16"/>
+      <c r="Z10" s="16">
+        <v>32.0</v>
+      </c>
       <c r="AA10" s="14">
         <f t="shared" si="1"/>
-        <v>249</v>
+        <v>281</v>
       </c>
     </row>
     <row r="11">
@@ -1472,10 +1480,12 @@
         <v>35.0</v>
       </c>
       <c r="Y11" s="12"/>
-      <c r="Z11" s="16"/>
+      <c r="Z11" s="16">
+        <v>37.0</v>
+      </c>
       <c r="AA11" s="14">
         <f t="shared" si="1"/>
-        <v>369</v>
+        <v>406</v>
       </c>
     </row>
     <row r="12">
@@ -1525,7 +1535,7 @@
       <c r="W12" s="12"/>
       <c r="X12" s="13"/>
       <c r="Y12" s="12"/>
-      <c r="Z12" s="18"/>
+      <c r="Z12" s="16"/>
       <c r="AA12" s="14">
         <f t="shared" si="1"/>
         <v>334</v>
@@ -1572,10 +1582,12 @@
       <c r="W13" s="12"/>
       <c r="X13" s="14"/>
       <c r="Y13" s="12"/>
-      <c r="Z13" s="16"/>
+      <c r="Z13" s="16">
+        <v>30.0</v>
+      </c>
       <c r="AA13" s="14">
         <f t="shared" si="1"/>
-        <v>193</v>
+        <v>223</v>
       </c>
     </row>
     <row r="14">
@@ -1637,7 +1649,7 @@
         <v>34.0</v>
       </c>
       <c r="Y14" s="12"/>
-      <c r="Z14" s="18"/>
+      <c r="Z14" s="16"/>
       <c r="AA14" s="14">
         <f t="shared" si="1"/>
         <v>528</v>
@@ -1700,17 +1712,19 @@
         <v>26.0</v>
       </c>
       <c r="Y15" s="12"/>
-      <c r="Z15" s="18"/>
+      <c r="Z15" s="16">
+        <v>34.0</v>
+      </c>
       <c r="AA15" s="14">
         <f t="shared" si="1"/>
-        <v>454</v>
+        <v>488</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="C16" s="18">
+      <c r="C16" s="16">
         <v>26.0</v>
       </c>
       <c r="D16" s="13"/>
@@ -1751,10 +1765,12 @@
       <c r="W16" s="20"/>
       <c r="X16" s="14"/>
       <c r="Y16" s="15"/>
-      <c r="Z16" s="16"/>
+      <c r="Z16" s="16">
+        <v>27.0</v>
+      </c>
       <c r="AA16" s="14">
         <f t="shared" si="1"/>
-        <v>276</v>
+        <v>303</v>
       </c>
     </row>
     <row r="17">
@@ -1909,7 +1925,9 @@
       <c r="Y19" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="Z19" s="24"/>
+      <c r="Z19" s="24" t="s">
+        <v>57</v>
+      </c>
       <c r="AA19" s="25"/>
     </row>
     <row r="20">
@@ -1975,7 +1993,9 @@
       <c r="Y20" s="27">
         <v>31.0</v>
       </c>
-      <c r="Z20" s="27"/>
+      <c r="Z20" s="27">
+        <v>37.0</v>
+      </c>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
@@ -2188,7 +2208,7 @@
       <c r="W5" s="15"/>
       <c r="X5" s="14"/>
       <c r="Y5" s="15"/>
-      <c r="Z5" s="16"/>
+      <c r="Z5" s="18"/>
       <c r="AA5" s="14">
         <f t="shared" ref="AA5:AA22" si="1">SUM(C5:Z5)</f>
         <v>50</v>
@@ -2239,10 +2259,12 @@
       <c r="Y6" s="12">
         <v>30.0</v>
       </c>
-      <c r="Z6" s="16"/>
+      <c r="Z6" s="16">
+        <v>33.0</v>
+      </c>
       <c r="AA6" s="14">
         <f t="shared" si="1"/>
-        <v>323</v>
+        <v>356</v>
       </c>
     </row>
     <row r="7">
@@ -2298,10 +2320,12 @@
       </c>
       <c r="X7" s="14"/>
       <c r="Y7" s="15"/>
-      <c r="Z7" s="16"/>
+      <c r="Z7" s="16">
+        <v>35.0</v>
+      </c>
       <c r="AA7" s="14">
         <f t="shared" si="1"/>
-        <v>379</v>
+        <v>414</v>
       </c>
     </row>
     <row r="8">
@@ -2347,10 +2371,12 @@
       </c>
       <c r="X8" s="14"/>
       <c r="Y8" s="12"/>
-      <c r="Z8" s="18"/>
+      <c r="Z8" s="16">
+        <v>24.0</v>
+      </c>
       <c r="AA8" s="14">
         <f t="shared" si="1"/>
-        <v>251</v>
+        <v>275</v>
       </c>
     </row>
     <row r="9">
@@ -2396,10 +2422,12 @@
         <v>35.0</v>
       </c>
       <c r="Y9" s="15"/>
-      <c r="Z9" s="16"/>
+      <c r="Z9" s="16">
+        <v>27.0</v>
+      </c>
       <c r="AA9" s="14">
         <f t="shared" si="1"/>
-        <v>267</v>
+        <v>294</v>
       </c>
     </row>
     <row r="10">
@@ -2443,7 +2471,7 @@
       </c>
       <c r="X10" s="13"/>
       <c r="Y10" s="15"/>
-      <c r="Z10" s="16"/>
+      <c r="Z10" s="18"/>
       <c r="AA10" s="14">
         <f t="shared" si="1"/>
         <v>231</v>
@@ -2492,10 +2520,12 @@
       <c r="Y11" s="12">
         <v>33.0</v>
       </c>
-      <c r="Z11" s="16"/>
+      <c r="Z11" s="16">
+        <v>38.0</v>
+      </c>
       <c r="AA11" s="14">
         <f t="shared" si="1"/>
-        <v>276</v>
+        <v>314</v>
       </c>
     </row>
     <row r="12">
@@ -2537,10 +2567,12 @@
       <c r="Y12" s="12">
         <v>31.0</v>
       </c>
-      <c r="Z12" s="18"/>
+      <c r="Z12" s="16">
+        <v>33.0</v>
+      </c>
       <c r="AA12" s="14">
         <f t="shared" si="1"/>
-        <v>197</v>
+        <v>230</v>
       </c>
     </row>
     <row r="13">
@@ -2590,10 +2622,12 @@
       </c>
       <c r="X13" s="14"/>
       <c r="Y13" s="12"/>
-      <c r="Z13" s="16"/>
+      <c r="Z13" s="16">
+        <v>36.0</v>
+      </c>
       <c r="AA13" s="14">
         <f t="shared" si="1"/>
-        <v>299</v>
+        <v>335</v>
       </c>
     </row>
     <row r="14">
@@ -2649,10 +2683,12 @@
       <c r="Y14" s="12">
         <v>30.0</v>
       </c>
-      <c r="Z14" s="16"/>
+      <c r="Z14" s="16">
+        <v>30.0</v>
+      </c>
       <c r="AA14" s="14">
         <f t="shared" si="1"/>
-        <v>386</v>
+        <v>416</v>
       </c>
     </row>
     <row r="15">
@@ -2708,10 +2744,12 @@
       <c r="Y15" s="12">
         <v>36.0</v>
       </c>
-      <c r="Z15" s="16"/>
+      <c r="Z15" s="16">
+        <v>35.0</v>
+      </c>
       <c r="AA15" s="14">
         <f t="shared" si="1"/>
-        <v>388</v>
+        <v>423</v>
       </c>
     </row>
     <row r="16">
@@ -2763,10 +2801,12 @@
         <v>26.0</v>
       </c>
       <c r="Y16" s="12"/>
-      <c r="Z16" s="16"/>
+      <c r="Z16" s="16">
+        <v>32.0</v>
+      </c>
       <c r="AA16" s="14">
         <f t="shared" si="1"/>
-        <v>327</v>
+        <v>359</v>
       </c>
     </row>
     <row r="17">
@@ -2820,10 +2860,12 @@
       </c>
       <c r="X17" s="13"/>
       <c r="Y17" s="12"/>
-      <c r="Z17" s="16"/>
+      <c r="Z17" s="16">
+        <v>36.0</v>
+      </c>
       <c r="AA17" s="14">
         <f t="shared" si="1"/>
-        <v>392</v>
+        <v>428</v>
       </c>
     </row>
     <row r="18">
@@ -2871,10 +2913,12 @@
       <c r="Y18" s="12">
         <v>38.0</v>
       </c>
-      <c r="Z18" s="18"/>
+      <c r="Z18" s="16">
+        <v>37.0</v>
+      </c>
       <c r="AA18" s="14">
         <f t="shared" si="1"/>
-        <v>306</v>
+        <v>343</v>
       </c>
     </row>
     <row r="19">
@@ -2936,10 +2980,12 @@
       <c r="Y19" s="12">
         <v>38.0</v>
       </c>
-      <c r="Z19" s="16"/>
+      <c r="Z19" s="16">
+        <v>36.0</v>
+      </c>
       <c r="AA19" s="14">
         <f t="shared" si="1"/>
-        <v>522</v>
+        <v>558</v>
       </c>
     </row>
     <row r="20">
@@ -2995,10 +3041,12 @@
       <c r="Y20" s="12">
         <v>31.0</v>
       </c>
-      <c r="Z20" s="18"/>
+      <c r="Z20" s="16">
+        <v>24.0</v>
+      </c>
       <c r="AA20" s="14">
         <f t="shared" si="1"/>
-        <v>387</v>
+        <v>411</v>
       </c>
     </row>
     <row r="21">
@@ -3042,10 +3090,12 @@
       </c>
       <c r="X21" s="14"/>
       <c r="Y21" s="15"/>
-      <c r="Z21" s="18"/>
+      <c r="Z21" s="16">
+        <v>30.0</v>
+      </c>
       <c r="AA21" s="14">
         <f t="shared" si="1"/>
-        <v>186</v>
+        <v>216</v>
       </c>
     </row>
     <row r="22">
@@ -3087,7 +3137,7 @@
       <c r="W22" s="12"/>
       <c r="X22" s="13"/>
       <c r="Y22" s="12"/>
-      <c r="Z22" s="18"/>
+      <c r="Z22" s="16"/>
       <c r="AA22" s="14">
         <f t="shared" si="1"/>
         <v>193</v>
@@ -3192,7 +3242,9 @@
       <c r="Y24" s="24" t="s">
         <v>99</v>
       </c>
-      <c r="Z24" s="24"/>
+      <c r="Z24" s="24" t="s">
+        <v>94</v>
+      </c>
       <c r="AA24" s="29"/>
     </row>
     <row r="25">
@@ -3256,7 +3308,9 @@
       <c r="Y25" s="27">
         <v>38.0</v>
       </c>
-      <c r="Z25" s="27"/>
+      <c r="Z25" s="27">
+        <v>38.0</v>
+      </c>
       <c r="AA25" s="14"/>
     </row>
   </sheetData>
@@ -3311,7 +3365,7 @@
       </c>
       <c r="B4" s="33"/>
       <c r="C4" s="34">
-        <v>7.0</v>
+        <v>6.0</v>
       </c>
     </row>
     <row r="5">
@@ -3329,7 +3383,7 @@
       </c>
       <c r="B6" s="33"/>
       <c r="C6" s="34">
-        <v>18.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="7">
@@ -3338,7 +3392,7 @@
       </c>
       <c r="B7" s="33"/>
       <c r="C7" s="34">
-        <v>11.0</v>
+        <v>10.0</v>
       </c>
     </row>
     <row r="8">
@@ -3401,7 +3455,7 @@
       </c>
       <c r="B14" s="33"/>
       <c r="C14" s="34">
-        <v>31.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="15">
@@ -7673,8 +7727,12 @@
       <c r="A25" s="13">
         <v>24.0</v>
       </c>
-      <c r="B25" s="44"/>
-      <c r="C25" s="45"/>
+      <c r="B25" s="44" t="s">
+        <v>54</v>
+      </c>
+      <c r="C25" s="45" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="14"/>
@@ -13054,19 +13112,19 @@
       </c>
       <c r="B25" s="47" t="str">
         <f>'SUNDAY SINGLES'!Z24</f>
-        <v/>
-      </c>
-      <c r="C25" s="47" t="str">
+        <v>CHRIS DUFFY</v>
+      </c>
+      <c r="C25" s="47">
         <f>'SUNDAY SINGLES'!Z25</f>
-        <v/>
+        <v>38</v>
       </c>
       <c r="D25" s="48" t="str">
         <f>'THURSDAY SINGLES'!Z19</f>
-        <v/>
-      </c>
-      <c r="E25" s="47" t="str">
+        <v>JOHN ANTCLIFFE</v>
+      </c>
+      <c r="E25" s="47">
         <f>'THURSDAY SINGLES'!Z20</f>
-        <v/>
+        <v>37</v>
       </c>
     </row>
     <row r="26">

</xml_diff>